<commit_message>
Record verified consolidation and final founder planning checkpoint
</commit_message>
<xml_diff>
--- a/docs/product/Pumdoki_MasterTracker_V4.xlsx
+++ b/docs/product/Pumdoki_MasterTracker_V4.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6421955959de4969"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R20d0c0fdfeb14b24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R4cd1a1055c6f4d05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="R076da55cc33d442b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R1e27f58481f74e43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legacy Overview 2026-08-16" sheetId="6" r:id="R29640443d6f442fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="7" r:id="R87000df78c0e4744"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Roadmap" sheetId="8" r:id="Rd8f3a2a75f5648fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Tracker" sheetId="9" r:id="R0593aec6001b46a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Blocker Queue" sheetId="10" r:id="R00052de970b041f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Log" sheetId="11" r:id="R4e9f5169e21d4e63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Register" sheetId="12" r:id="R543c9fb70a2d4cc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Budget" sheetId="13" r:id="R0d00416ae27b4ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R463b69d9d498496b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R723d300d33c6492f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="Re3e41bcb8c174859"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="Rc9c5c67bfc244714"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R10f5e7b319bc4d5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legacy Overview 2026-08-16" sheetId="6" r:id="R5cba30f21af54714"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="7" r:id="R821888b8c9da4f22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Roadmap" sheetId="8" r:id="Rb66976c9c95344fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Tracker" sheetId="9" r:id="Refbf8927fd154fb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Blocker Queue" sheetId="10" r:id="Rbf04dc1fb8054323"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Log" sheetId="11" r:id="R6298a8167dd44592"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Register" sheetId="12" r:id="R7c354f8b579a4c9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Budget" sheetId="13" r:id="R7443d5d0881e4ea1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4678,7 +4678,7 @@
         <x:v>Latest merge</x:v>
       </x:c>
       <x:c r="H38" s="111" t="str">
-        <x:v>Slice 3: PR #15; Slice 4 reconciliation in HANDOFF.md</x:v>
+        <x:v>Slice 3: PR #15; Slice 4: PR #17 merged in dev 56cb0ad</x:v>
       </x:c>
       <x:c r="I38" s="111" t="str">
         <x:v>Next founder task</x:v>
@@ -5821,23 +5821,23 @@
         <x:v>Truthful prototype copy</x:v>
       </x:c>
       <x:c r="E5" s="111" t="str">
-        <x:v>Publish verified legal UI cleanup</x:v>
+        <x:v>Release verified legal UI cleanup</x:v>
       </x:c>
       <x:c r="F5" s="111" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="G5" s="111" t="str">
         <x:v>Engineering</x:v>
       </x:c>
       <x:c r="H5" s="111" t="str">
-        <x:v>Publication checks</x:v>
+        <x:v>Approved website release</x:v>
       </x:c>
       <x:c r="I5" s="111" t="str">
-        <x:v>Local cleanup verified: web219/contracts24/non-database API273 and builds passed. See HANDOFF.md for release proof; final counsel copy remains future work.</x:v>
+        <x:v>Cleanup source is pushed to dev in 56cb0ad. Deploy in an approved website release; final counsel policies and actual processes remain future work. CI/main evidence is in HANDOFF.md.</x:v>
       </x:c>
       <x:c r="J5" s="112"/>
       <x:c r="K5" s="111" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/PLAN.md</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/commit/56cb0adaffa4896aa9d54257b4eecfe18804bb54</x:v>
       </x:c>
       <x:c r="L5" s="112" t="n">
         <x:v>46271.666666666664</x:v>
@@ -5857,19 +5857,17 @@
         <x:v>Branch reconciliation</x:v>
       </x:c>
       <x:c r="E6" s="111" t="str">
-        <x:v>Publish locally integrated Slice 4 source</x:v>
+        <x:v>Slice 4 source published to dev</x:v>
       </x:c>
       <x:c r="F6" s="111" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G6" s="111" t="str">
         <x:v>Engineering</x:v>
       </x:c>
-      <x:c r="H6" s="111" t="str">
-        <x:v>Publication checks</x:v>
-      </x:c>
+      <x:c r="H6" s="111"/>
       <x:c r="I6" s="111" t="str">
-        <x:v>PR17 source25057bd integrated locally with317abda ancestry. Original CI33337682290 green; final current-head publication checks recorded in HANDOFF.md.</x:v>
+        <x:v>PR #17 merged through dev 56cb0ad, preserving 317abda/25057bd ancestry. Final CI and main-publication evidence is in HANDOFF.md; no deployment or operations activation is implied.</x:v>
       </x:c>
       <x:c r="J6" s="112"/>
       <x:c r="K6" s="111" t="str">
@@ -5959,7 +5957,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6bac1ca91f24b1b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R279de878b6de4fc5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7057,7 +7055,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e632e6626a8499c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb0ebf8501b84402"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7529,7 +7527,7 @@
         <x:v>Slice 3 merged in PR #15. Provider-neutral dormant foundation exists; no operational provider/session/hosting activation. G1–G12 remain NOT EVALUATED.</x:v>
       </x:c>
       <x:c r="H16" s="111" t="str">
-        <x:v>Park additional operations work while founder completes the initial business definition. Confirm current Slice 4 integration in HANDOFF.md; production activation stays separately evaluated.</x:v>
+        <x:v>Park additional operations work while founder completes the initial business definition. Slice 4 source is pushed to dev in 56cb0ad and PR #17 is merged. Final CI/main evidence is in HANDOFF.md; activation remains separate.</x:v>
       </x:c>
       <x:c r="I16" s="111" t="str">
         <x:v>https://github.com/QK-Connoisseur/PDoki/pull/15</x:v>
@@ -7858,13 +7856,13 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="G27" s="173" t="str">
-        <x:v>Truthful prototype legal cleanup complete locally; web219, contracts24 and non-database API273 tests and builds passed. Production policies and processes remain unfinished.</x:v>
+        <x:v>Truthful prototype legal cleanup is pushed to dev in 56cb0ad. Local web219, contracts24, non-database API273 and builds passed. Production policies and processes remain unfinished.</x:v>
       </x:c>
       <x:c r="H27" s="173" t="str">
         <x:v>Ship truthful placeholder copy with the next approved website release. Before public launch, counsel approves final policies and operators verify actual contacts/processes; deployment is separate from a Git merge.</x:v>
       </x:c>
       <x:c r="I27" s="173" t="str">
-        <x:v>September 6, 2026 local verification; HANDOFF.md for publication evidence</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/commit/56cb0adaffa4896aa9d54257b4eecfe18804bb54</x:v>
       </x:c>
       <x:c r="J27" s="174" t="n">
         <x:v>46271.666666666664</x:v>
@@ -7894,7 +7892,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6baf1d96d7624d96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbae23f22bfbd44ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18964,7 +18962,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra367d6caad5d49e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f8bb2389d85457d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26662,7 +26660,7 @@
       </x:c>
       <x:c r="N149" s="112"/>
       <x:c r="O149" s="111" t="str">
-        <x:v>HANDOFF.md — September 6, 2026: web219/contracts24/non-database API273 and builds passed</x:v>
+        <x:v>https://github.com/QK-Connoisseur/PDoki/commit/56cb0adaffa4896aa9d54257b4eecfe18804bb54</x:v>
       </x:c>
       <x:c r="P149" s="112" t="n">
         <x:v>46271.666666666664</x:v>
@@ -26671,7 +26669,7 @@
         <x:v>Replace unconfigured production-looking emails with .example sample addresses until real domains and mailboxes are operational.</x:v>
       </x:c>
       <x:c r="R149" s="111" t="str">
-        <x:v>Prototype legal claims and unconfigured production-looking contacts corrected locally. Source integration does not deploy the website or establish final operating policies.</x:v>
+        <x:v>Prototype legal claims and unconfigured production-looking contacts corrected and pushed to dev in 56cb0ad. Final CI/main publication evidence is in HANDOFF.md. A source merge does not deploy the website or establish final policies.</x:v>
       </x:c>
       <x:c r="S149" s="111" t="str">
         <x:v>Preserved Master Tracker row 162; legacy status: 📋 Not Started</x:v>
@@ -27529,7 +27527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a16687151ed4743"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79e8f6906de846af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record Maryland LLC filing and sent CCBill inquiry
</commit_message>
<xml_diff>
--- a/docs/product/Pumdoki_MasterTracker_V4.xlsx
+++ b/docs/product/Pumdoki_MasterTracker_V4.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R463b69d9d498496b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R723d300d33c6492f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="Re3e41bcb8c174859"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="Rc9c5c67bfc244714"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R10f5e7b319bc4d5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legacy Overview 2026-08-16" sheetId="6" r:id="R5cba30f21af54714"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="7" r:id="R821888b8c9da4f22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Roadmap" sheetId="8" r:id="Rb66976c9c95344fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Tracker" sheetId="9" r:id="Refbf8927fd154fb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Blocker Queue" sheetId="10" r:id="Rbf04dc1fb8054323"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Log" sheetId="11" r:id="R6298a8167dd44592"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Register" sheetId="12" r:id="R7c354f8b579a4c9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Budget" sheetId="13" r:id="R7443d5d0881e4ea1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7795711c1c2c4fd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R2044898aa65d4e38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R404a5f97f40147d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="Rb807e3ab990a40b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R7bfc52ffe2bc40f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legacy Overview 2026-08-16" sheetId="6" r:id="R9494421699b1422d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="7" r:id="R362a974d66b74322"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Roadmap" sheetId="8" r:id="R8c78190525054a80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Tracker" sheetId="9" r:id="R778bb3c34800408b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Blocker Queue" sheetId="10" r:id="Rd242103954474179"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Log" sheetId="11" r:id="R429c6bd7ab0245a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Register" sheetId="12" r:id="R8635ba7f128346ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Budget" sheetId="13" r:id="Rd60094f2100c445e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3379,7 +3379,7 @@
     </x:row>
     <x:row r="2" ht="21.75" customHeight="1">
       <x:c r="A2" s="92" t="str">
-        <x:v>Refreshed September 6, 2026. Start with the initial business definition. Record counts are navigation metrics, not launch readiness.</x:v>
+        <x:v>Updated September 8, 2026. Founder reports LLC filed and CCBill sales inquiry sent. Await responses. Record counts are navigation metrics, not launch readiness.</x:v>
       </x:c>
       <x:c r="B2" s="92"/>
       <x:c r="C2" s="92"/>
@@ -3421,12 +3421,12 @@
         <x:v>Phase</x:v>
       </x:c>
       <x:c r="B5" s="109" t="str">
-        <x:v>P00 — Initial business definition</x:v>
+        <x:v>P06 — Await CCBill sales response</x:v>
       </x:c>
       <x:c r="D5"/>
       <x:c r="E5"/>
       <x:c r="I5" s="130" t="str">
-        <x:v>Complete the one-page initial business definition. This is the only founder assignment now; no purchase is required.</x:v>
+        <x:v>Founder reports Kiban Digital Holdings LLC filed in Maryland and preliminary inquiry sent to CCBill sales. Await state approval and sales response. Next: share and review the response when received. No duplicate inquiry or new founder assignment.</x:v>
       </x:c>
       <x:c r="J5" s="130"/>
       <x:c r="K5" s="130"/>
@@ -3439,7 +3439,7 @@
         <x:v>Work</x:v>
       </x:c>
       <x:c r="B6" s="111" t="str">
-        <x:v>Founder definition and current instruction reconciliation</x:v>
+        <x:v>Await Maryland and CCBill responses</x:v>
       </x:c>
       <x:c r="D6"/>
       <x:c r="E6"/>
@@ -3486,7 +3486,7 @@
         <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/PLAN.md</x:v>
       </x:c>
       <x:c r="I9" s="131" t="str">
-        <x:v>Use Launch Budget for current funding. $1,000–$5,000 is available now; another $5,000 is possible and uncommitted. Local CI or a Git merge does not establish launch readiness or deploy the site.</x:v>
+        <x:v>Funding notes: founder reports a $1,800 monthly ceiling; this is not lump-sum cash or funded runway. Existing $1,000–$5,000 cash assumptions remain until clarified. See Launch Budget.</x:v>
       </x:c>
       <x:c r="J9" s="131"/>
       <x:c r="K9" s="131"/>
@@ -3556,7 +3556,7 @@
       <x:c r="D13" s="151"/>
       <x:c r="E13" s="150" t="n">
         <x:f>COUNTIF('Delivery Tracker'!$H$4:$H$400,"In Progress")</x:f>
-        <x:v>49</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="F13" s="151"/>
       <x:c r="G13" s="150" t="n">
@@ -3571,7 +3571,7 @@
       <x:c r="J13" s="151"/>
       <x:c r="K13" s="150" t="n">
         <x:f>COUNTIF('Delivery Tracker'!$H$4:$H$400,"Not Started")</x:f>
-        <x:v>78</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="L13" s="151"/>
       <x:c r="M13" s="158" t="n">
@@ -3925,7 +3925,7 @@
       </x:c>
       <x:c r="H22" s="111" t="n">
         <x:f>'Phase Roadmap'!H8</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="I22" s="111" t="n">
         <x:f>'Phase Roadmap'!I8</x:f>
@@ -3937,11 +3937,11 @@
       </x:c>
       <x:c r="K22" s="111" t="n">
         <x:f>'Phase Roadmap'!K8</x:f>
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="L22" s="111" t="str">
         <x:f>'Phase Roadmap'!L8</x:f>
-        <x:v>Slices 1–3 are published, including PR #15. The private router remains dormant. Founder business definition is the next active task.</x:v>
+        <x:v>Slices 1–4 have published source; operations remain dormant. Founder reports Maryland LLC filed and CCBill inquiry sent. Await approval/response; review what arrives before another founder task.</x:v>
       </x:c>
       <x:c r="M22" s="111" t="str">
         <x:f>'Phase Roadmap'!M8</x:f>
@@ -4347,7 +4347,7 @@
       </x:c>
       <x:c r="L29" s="111" t="str">
         <x:f>'Phase Roadmap'!L15</x:f>
-        <x:v>Slice 3 is published in PR #15. Dormant private-operations foundation remains; further work is parked during founder business definition.</x:v>
+        <x:v>Dormant operations foundation has published source. Further operations work stays parked while Maryland approval and CCBill sales response are pending.</x:v>
       </x:c>
       <x:c r="M29" s="111" t="str">
         <x:f>'Phase Roadmap'!M15</x:f>
@@ -4556,7 +4556,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B35" s="109" t="str">
-        <x:v>Start with the one-page initial business definition; review other decisions only when they become the next step.</x:v>
+        <x:v>LLC filed and CCBill inquiry sent, per founder report. Wait for Maryland approval and CCBill sales response. Review the response when received, then choose one next action.</x:v>
       </x:c>
       <x:c r="C35" s="109" t="str">
         <x:v>2</x:v>
@@ -4684,7 +4684,7 @@
         <x:v>Next founder task</x:v>
       </x:c>
       <x:c r="J38" s="111" t="str">
-        <x:v>Complete the initial business definition.</x:v>
+        <x:v>Share and review Maryland/CCBill responses when received.</x:v>
       </x:c>
       <x:c r="K38" s="111" t="str"/>
       <x:c r="L38" s="111" t="str"/>
@@ -5773,38 +5773,38 @@
     </x:row>
     <x:row r="4" ht="54" customHeight="1">
       <x:c r="A4" s="109" t="str">
-        <x:v>DEC-SEQUENTIAL</x:v>
+        <x:v>DEC-CCBILL</x:v>
       </x:c>
       <x:c r="B4" s="109" t="str">
-        <x:v>P00</x:v>
+        <x:v>P06</x:v>
       </x:c>
       <x:c r="C4" s="109" t="str">
-        <x:v>Baseline, tracker, and scope control</x:v>
+        <x:v>Wallet, payments and payouts</x:v>
       </x:c>
       <x:c r="D4" s="109" t="str">
-        <x:v>Founder definition</x:v>
+        <x:v>Await processor response</x:v>
       </x:c>
       <x:c r="E4" s="109" t="str">
-        <x:v>Complete the one-page initial business definition</x:v>
+        <x:v>Review CCBill response when received</x:v>
       </x:c>
       <x:c r="F4" s="109" t="str">
-        <x:v>Ready</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="G4" s="109" t="str">
         <x:v>Founder</x:v>
       </x:c>
       <x:c r="H4" s="109" t="str">
-        <x:v>Founder</x:v>
+        <x:v>Awaiting CCBill sales response</x:v>
       </x:c>
       <x:c r="I4" s="109" t="str">
-        <x:v>Fill the template. This is the only active founder assignment; $0 spending.</x:v>
+        <x:v>Founder reports CCBill sales inquiry sent and Maryland LLC filed. Wait for sales response and state approval; share/review what arrives before the next founder action. No reply or approval evidenced.</x:v>
       </x:c>
       <x:c r="J4" s="110"/>
       <x:c r="K4" s="109" t="str">
-        <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/PLAN.md</x:v>
+        <x:v>docs/product/initial-ccbill-inquiry.md</x:v>
       </x:c>
       <x:c r="L4" s="110" t="n">
-        <x:v>46271.666666666664</x:v>
+        <x:v>46273.666666666664</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="54" customHeight="1">
@@ -5957,7 +5957,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R279de878b6de4fc5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9807d8f6f37d41c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7055,7 +7055,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb0ebf8501b84402"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48a368095cad4ec5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7285,7 +7285,7 @@
         <x:v>Local Mailpit and provider-neutral mail exist. Production startup correctly fails closed without approved delivery.</x:v>
       </x:c>
       <x:c r="H8" s="111" t="str">
-        <x:v>Choose email after business definition, counsel/entity and processor fit, country/data boundaries and funded staging scope. Then configure/test verified sender, SPF/DKIM/DMARC, bounce/complaint handling and deliverability before external account flows.</x:v>
+        <x:v>Choose email after entity, processor fit, country/data boundaries and funded staging scope are known. Configure and test sender authentication, bounce handling and delivery before external account flows.</x:v>
       </x:c>
       <x:c r="I8" s="111" t="str">
         <x:v>https://github.com/QK-Connoisseur/PDoki/tree/dev/docs/operations</x:v>
@@ -7302,26 +7302,26 @@
         <x:v>P04</x:v>
       </x:c>
       <x:c r="C9" s="111" t="str">
-        <x:v>LLC attorney/CPA shortlist and entity state</x:v>
+        <x:v>Maryland LLC filed; approval pending</x:v>
       </x:c>
       <x:c r="D9" s="111" t="str">
         <x:v>Founder</x:v>
       </x:c>
-      <x:c r="E9" s="112" t="n">
-        <x:v>46233.666666666664</x:v>
-      </x:c>
+      <x:c r="E9" s="112"/>
       <x:c r="F9" s="111" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="G9" s="111" t="str">
-        <x:v>No entity is filed.</x:v>
+        <x:v>Founder reports Kiban Digital Holdings LLC filed in Maryland through Northwest; state approval pending. Exact filing date, filing ID, EIN, bank account and actual cost have not been supplied.</x:v>
       </x:c>
       <x:c r="H9" s="111" t="str">
-        <x:v>Obtain qualified privacy-focused adult-platform legal and tax advice.</x:v>
-      </x:c>
-      <x:c r="I9" s="111" t="str"/>
+        <x:v>Await Maryland approval and approved formation documents. Record invoice when available. Next founder action is to share and review the received Maryland or CCBill response.</x:v>
+      </x:c>
+      <x:c r="I9" s="111" t="str">
+        <x:v>Founder report, September 8, 2026: LLC filed and CCBill sales inquiry sent. Exact event times, state approval and processor response not supplied.</x:v>
+      </x:c>
       <x:c r="J9" s="112" t="n">
-        <x:v>46255.666666666664</x:v>
+        <x:v>46273.666666666664</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="55" customHeight="1">
@@ -7332,26 +7332,26 @@
         <x:v>P06</x:v>
       </x:c>
       <x:c r="C10" s="111" t="str">
-        <x:v>CCBill requirements and fee quote</x:v>
+        <x:v>Preliminary CCBill model fit and costs</x:v>
       </x:c>
       <x:c r="D10" s="111" t="str">
         <x:v>Founder</x:v>
       </x:c>
-      <x:c r="E10" s="112" t="n">
-        <x:v>46233.666666666664</x:v>
-      </x:c>
+      <x:c r="E10" s="112"/>
       <x:c r="F10" s="111" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="G10" s="111" t="str">
-        <x:v>Merchant application and concrete pricing have not started.</x:v>
+        <x:v>Founder reports the preliminary inquiry was sent to CCBill sales. No reply, quote, formal merchant approval or activation is evidenced. Epoch remains a possible later provider.</x:v>
       </x:c>
       <x:c r="H10" s="111" t="str">
-        <x:v>Request the merchant package, technical documents, and complete fee quote.</x:v>
-      </x:c>
-      <x:c r="I10" s="111" t="str"/>
+        <x:v>Await and review the sales response for model eligibility, countries, Veso, creator payouts, complete fees/reserves and required documents. Do not send a duplicate inquiry or assume approval.</x:v>
+      </x:c>
+      <x:c r="I10" s="111" t="str">
+        <x:v>Founder report, September 8, 2026: LLC filed and CCBill sales inquiry sent. Exact event times, state approval and processor response not supplied.</x:v>
+      </x:c>
       <x:c r="J10" s="112" t="n">
-        <x:v>46255.666666666664</x:v>
+        <x:v>46273.666666666664</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="55" customHeight="1">
@@ -7434,12 +7434,14 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G13" s="111" t="str">
-        <x:v>Payment, payout, identity, adult-content law, privacy, tax, sanctions, and support coverage remain open.</x:v>
+        <x:v>Operating location is confirmed as Maryland, USA. Creator/member countries remain unanswered; eligibility and service coverage remain unresolved.</x:v>
       </x:c>
       <x:c r="H13" s="111" t="str">
-        <x:v>Start with the US and only supported Latin American countries after review.</x:v>
-      </x:c>
-      <x:c r="I13" s="111" t="str"/>
+        <x:v>Use CCBill eligibility to narrow proposed creator/member countries. Obtain targeted legal review of unresolved country obligations before real launch.</x:v>
+      </x:c>
+      <x:c r="I13" s="111" t="str">
+        <x:v>docs/product/initial-business-definition.md — founder answers reviewed September 6, 2026</x:v>
+      </x:c>
       <x:c r="J13" s="112" t="n">
         <x:v>46255.666666666664</x:v>
       </x:c>
@@ -7464,12 +7466,14 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G14" s="111" t="str">
-        <x:v>Veso remains. Proposed founding cohort ~500 pays necessary processing fees only; platform commission duration, fee definition, refunds/reserves, payouts and Plus revenue remain unresolved.</x:v>
+        <x:v>Founder corrected the offer: Pumdoki should recover costs without profit on founding creator sales. Processing-fees-only is superseded. Duration, fee allocation and no-loss economics are unproven.</x:v>
       </x:c>
       <x:c r="H14" s="111" t="str">
-        <x:v>Use written processor terms to model a fees-only cohort. Zero platform commission provides no contribution toward operations before other revenue.</x:v>
-      </x:c>
-      <x:c r="I14" s="111" t="str"/>
+        <x:v>After counsel/processor fit, define attributable costs, refunds, chargebacks, reserves and payout allocation before quoting founder fees. No loss-free promise is supported yet.</x:v>
+      </x:c>
+      <x:c r="I14" s="111" t="str">
+        <x:v>docs/product/initial-business-definition.md — founder answers reviewed September 6, 2026</x:v>
+      </x:c>
       <x:c r="J14" s="112" t="n">
         <x:v>46271.666666666664</x:v>
       </x:c>
@@ -7527,7 +7531,7 @@
         <x:v>Slice 3 merged in PR #15. Provider-neutral dormant foundation exists; no operational provider/session/hosting activation. G1–G12 remain NOT EVALUATED.</x:v>
       </x:c>
       <x:c r="H16" s="111" t="str">
-        <x:v>Park additional operations work while founder completes the initial business definition. Slice 4 source is pushed to dev in 56cb0ad and PR #17 is merged. Final CI/main evidence is in HANDOFF.md; activation remains separate.</x:v>
+        <x:v>Operations work stays parked while awaiting CCBill response. Slice 4 is published; final CI/main evidence is in HANDOFF.md. Deployment and activation remain separate.</x:v>
       </x:c>
       <x:c r="I16" s="111" t="str">
         <x:v>https://github.com/QK-Connoisseur/PDoki/pull/15</x:v>
@@ -7606,26 +7610,26 @@
         <x:v>P00</x:v>
       </x:c>
       <x:c r="C19" s="173" t="str">
-        <x:v>One founder task at a time</x:v>
+        <x:v>Initial business definition and sequential workflow</x:v>
       </x:c>
       <x:c r="D19" s="173" t="str">
         <x:v>Founder</x:v>
       </x:c>
       <x:c r="E19" s="173"/>
       <x:c r="F19" s="173" t="str">
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G19" s="173" t="str">
-        <x:v>Founder has limited time. Work is sequential; no parallel founder assignments.</x:v>
+        <x:v>Business definition answered/reviewed and operating location confirmed as Maryland, USA. Work remains sequential, one founder assignment at a time.</x:v>
       </x:c>
       <x:c r="H19" s="173" t="str">
-        <x:v>Complete the one-page initial business definition next. No purchases required.</x:v>
+        <x:v>Current: await Maryland approval and CCBill sales response. Founder reports filing and inquiry completed. Share/review the response when received, then choose one next action.</x:v>
       </x:c>
       <x:c r="I19" s="173" t="str">
-        <x:v>Founder decision, September 6, 2026</x:v>
+        <x:v>Founder report, September 8, 2026: LLC filed and CCBill sales inquiry sent. Exact event times, state approval and processor response not supplied.</x:v>
       </x:c>
       <x:c r="J19" s="174" t="n">
-        <x:v>46271.666666666664</x:v>
+        <x:v>46273.666666666664</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="95" customHeight="1">
@@ -7736,13 +7740,13 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="G23" s="173" t="str">
-        <x:v>Target around 500 founding creators; necessary processing fees only and founder profile tag. Recruitment relationship via former Epal contact and Discord servers.</x:v>
+        <x:v>Two contacts could help recruit 50–100 creators; these are prospects, not commitments. Founder badge and cost recovery with no profit on founder sales remain the direction. About 500 is a longer target.</x:v>
       </x:c>
       <x:c r="H23" s="173" t="str">
-        <x:v>Define eligibility, number, duration and covered fees. Validate unit economics before making public commitments.</x:v>
+        <x:v>Define first-cohort eligibility, countries, duration and cost allocation after counsel/processor fit. No-loss economics and Plus/top 100 benefits remain unproven.</x:v>
       </x:c>
       <x:c r="I23" s="173" t="str">
-        <x:v>Founder direction, September 6, 2026; commercial terms provisional</x:v>
+        <x:v>docs/product/initial-business-definition.md — founder answers reviewed September 6, 2026</x:v>
       </x:c>
       <x:c r="J23" s="174" t="n">
         <x:v>46271.666666666664</x:v>
@@ -7796,16 +7800,16 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="G25" s="173" t="str">
-        <x:v>Available now: $1,000–$5,000 total. Another $5,000 may become available over coming months; it is uncommitted. No expense was recorded as paid.</x:v>
+        <x:v>Founder now reports a $1,800 monthly ceiling and proposed recruiter/helper $300–$400/month. Inclusion in that ceiling and overlap with budget backup allowance are unconfirmed. Earlier cash assumptions remain.</x:v>
       </x:c>
       <x:c r="H25" s="173" t="str">
-        <x:v>Use Launch Budget. First step costs $0; seek and approve one scoped quote at a time after the definition.</x:v>
+        <x:v>Keep cost allowances until actual quotes/invoices support changes. LLC filing is reported but amount/payment details were not supplied; actual cost remains blank. Monthly funding and helper overlap remain unresolved.</x:v>
       </x:c>
       <x:c r="I25" s="173" t="str">
-        <x:v>Founder funding statement, September 6, 2026; docs/product/launch-budget.md</x:v>
+        <x:v>Founder funding statements September 6 and filed-LLC/sent-inquiry report September 8, 2026</x:v>
       </x:c>
       <x:c r="J25" s="174" t="n">
-        <x:v>46271.666666666664</x:v>
+        <x:v>46273.666666666664</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="95" customHeight="1">
@@ -7826,16 +7830,16 @@
         <x:v>Ready</x:v>
       </x:c>
       <x:c r="G26" s="173" t="str">
-        <x:v>Fiverr may source technical reviewers. Relevant experience, written scope, findings and a retest matter more than marketplace or low price.</x:v>
+        <x:v>Use DIY work, suitable Fiverr specialists and drafts to control cost. Necessary legal work uses a qualified lawyer reviewing the actual model. Record the reviewed version, corrections and remaining limitations.</x:v>
       </x:c>
       <x:c r="H26" s="173" t="str">
-        <x:v>Counsel discovery after definition; architecture/ledger/entitlement review before money/media design locks; independent integrated review and retest before real users, identity, content or money.</x:v>
+        <x:v>Buy targeted legal advice only for unresolved requirements or necessary document/workflow review. Technical design review precedes fixed money/media designs; independent integrated assessment and retest precede real launch.</x:v>
       </x:c>
       <x:c r="I26" s="173" t="str">
-        <x:v>Founder direction and staged budget, September 6, 2026</x:v>
+        <x:v>Founder instruction, September 8, 2026</x:v>
       </x:c>
       <x:c r="J26" s="174" t="n">
-        <x:v>46271.666666666664</x:v>
+        <x:v>46273.666666666664</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="95" customHeight="1">
@@ -7892,7 +7896,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbae23f22bfbd44ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45740b3e98174502"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7917,7 +7921,7 @@
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="177" t="str">
-        <x:v>September 6, 2026</x:v>
+        <x:v>September 8, 2026</x:v>
       </x:c>
       <x:c r="B2" s="179"/>
       <x:c r="C2" s="179"/>
@@ -7956,7 +7960,7 @@
         <x:v>5000</x:v>
       </x:c>
       <x:c r="D5" s="177" t="str">
-        <x:v>Founder total cash range, not a monthly allowance.</x:v>
+        <x:v>Earlier total-cash assumption retained. New user-reported $1,800 monthly ceiling is not lump-sum cash or funded runway; sustainability is unconfirmed.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="32" customHeight="1">
@@ -8121,12 +8125,12 @@
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
       <x:c r="A17" s="177" t="str">
-        <x:v>Next action costs $0</x:v>
+        <x:v>Current: await CCBill response</x:v>
       </x:c>
       <x:c r="B17" s="179"/>
       <x:c r="C17" s="179"/>
       <x:c r="D17" s="177" t="str">
-        <x:v>Complete the initial business definition. Then seek one scoped counsel consultation with a spending cap you approve.</x:v>
+        <x:v>Founder reports Kiban Digital Holdings LLC filed in Maryland and preliminary inquiry sent to CCBill sales. Await state approval and sales response; review what arrives before another founder task.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="64" customHeight="1">
@@ -8136,7 +8140,7 @@
       <x:c r="B18" s="179"/>
       <x:c r="C18" s="179"/>
       <x:c r="D18" s="177" t="str">
-        <x:v>25 invited creators, founder runs moderation/support with paid backup allowance. 500 creators is an aspiration, not a day-one staffing or cost assumption.</x:v>
+        <x:v>Pilot counts remain planning assumptions. Two contacts may help recruit 50–100 creators; no committed cohort or creator/member countries were supplied.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="32" customHeight="1">
@@ -8161,7 +8165,7 @@
     </x:row>
     <x:row r="21" ht="48" customHeight="1">
       <x:c r="A21" s="177" t="str">
-        <x:v>Counsel discovery consultation</x:v>
+        <x:v>Targeted legal advice allowance</x:v>
       </x:c>
       <x:c r="B21" s="190" t="n">
         <x:v>300</x:v>
@@ -8170,12 +8174,12 @@
         <x:v>800</x:v>
       </x:c>
       <x:c r="D21" s="177" t="str">
-        <x:v>After definition. Adult-platform business, country and Veso fit. Unquoted scoped allowance.</x:v>
+        <x:v>Optional scoped advice for unresolved material issues. DIY/Fiverr drafts first where suitable; use a qualified lawyer when needed. Unquoted allowance unchanged; no legal engagement.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="48" customHeight="1">
       <x:c r="A22" s="177" t="str">
-        <x:v>CPA / entity consultation</x:v>
+        <x:v>Targeted tax / accounting advice</x:v>
       </x:c>
       <x:c r="B22" s="190" t="n">
         <x:v>100</x:v>
@@ -8184,12 +8188,12 @@
         <x:v>300</x:v>
       </x:c>
       <x:c r="D22" s="177" t="str">
-        <x:v>After counsel direction. Entity, banking, tax and records scope. Unquoted.</x:v>
+        <x:v>Use when a specific tax or accounting question needs professional advice. Founder reports LLC filed; state approval pending. Unquoted allowance unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="48" customHeight="1">
       <x:c r="A23" s="200" t="str">
-        <x:v>Discovery subtotal</x:v>
+        <x:v>Initial advice allowances subtotal</x:v>
       </x:c>
       <x:c r="B23" s="201" t="n">
         <x:f>SUM(B21:B22)</x:f>
@@ -8200,7 +8204,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="D23" s="200" t="str">
-        <x:v>Do not spend the whole available budget on build work before these answers.</x:v>
+        <x:v>Reserve for necessary questions. This is not a required discovery purchase or a commitment to spend.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="48" customHeight="1">
@@ -8214,12 +8218,12 @@
         <x:v>900</x:v>
       </x:c>
       <x:c r="D24" s="177" t="str">
-        <x:v>Only after advice; jurisdiction and registered-agent/filing costs are unknown. Allowance.</x:v>
+        <x:v>Founder reports Maryland LLC filed through Northwest; state approval pending. Actual invoice and recurring charges not supplied; this allowance is not amount paid.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="48" customHeight="1">
       <x:c r="A25" s="177" t="str">
-        <x:v>Adult legal documents / consent</x:v>
+        <x:v>Legal document drafting / review</x:v>
       </x:c>
       <x:c r="B25" s="190" t="n">
         <x:v>2000</x:v>
@@ -8228,7 +8232,7 @@
         <x:v>6000</x:v>
       </x:c>
       <x:c r="D25" s="177" t="str">
-        <x:v>Before real activity. Qualified adult-platform counsel, usable scope and revisions; unquoted, not a guaranteed market minimum.</x:v>
+        <x:v>Prepare suitable drafts yourself or with Fiverr specialists; qualified adult-platform counsel reviews and corrects necessary final documents/workflows. Unquoted allowance unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="48" customHeight="1">
@@ -8488,7 +8492,7 @@
         <x:v>600</x:v>
       </x:c>
       <x:c r="D44" s="177" t="str">
-        <x:v>Unquoted limited-hours allowance. Founder supplies daily unpaid coverage; define capacity and qualified backup before any real activity. Not 24/7 staffing.</x:v>
+        <x:v>Proposed Discord recruiter/helper: $300–$400/month. Inclusion in $1,800 ceiling and overlap with this $100–$600 backup allowance are unconfirmed; no amount added. Scope/coverage remain unverified.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="48" customHeight="1">
@@ -8562,7 +8566,7 @@
       <x:c r="B51" s="179"/>
       <x:c r="C51" s="179"/>
       <x:c r="D51" s="177" t="str">
-        <x:v>Fees-only creators yield no platform commission to cover operations. Plus revenue is unproven and excluded. Define duration, necessary fees and who absorbs losses before promising benefits.</x:v>
+        <x:v>Founder correction: recover attributable costs without profit on founding creator sales. Processing-fees-only is superseded. Duration, cost allocation and no-loss economics are unproven; Plus revenue excluded.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="32" customHeight="1">
@@ -8596,7 +8600,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="D54" s="177" t="str">
-        <x:v>Planning assumption; ~500 is the longer recruitment target. Counts are not existing commitments.</x:v>
+        <x:v>Unchanged planning counts. Two contacts could recruit 50–100 prospects, not commitments; ~500 remains the longer target.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="64" customHeight="1">
@@ -8722,7 +8726,7 @@
       <x:c r="B66" s="179"/>
       <x:c r="C66" s="179"/>
       <x:c r="D66" s="177" t="str">
-        <x:v>Planning judgment, September 6, 2026. No lawyer, reviewer, provider or operator has quoted or accepted this scope.</x:v>
+        <x:v>Planning allowances remain unquoted. Founder answers reviewed September 6, 2026 in initial-business-definition.md; new funding/helper statements are notes only, not formula changes.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="64" customHeight="1">
@@ -8742,7 +8746,7 @@
       <x:c r="B68" s="179"/>
       <x:c r="C68" s="179"/>
       <x:c r="D68" s="177" t="str">
-        <x:v>After definition: one counsel discovery quote, then entity/processor fit and cash terms, then funded technical review/design. No paid platform, reward or production commitment implied.</x:v>
+        <x:v>Current: wait for Maryland approval and CCBill sales response, then review the response. DIY/Fiverr and targeted qualified review remain the approach. Costs/formulas unchanged; actual filing expense unknown.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="32" customHeight="1">
@@ -15334,7 +15338,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="13" t="str">
-        <x:v>Historical estimates only. Corrected arithmetic below; use Launch Budget for current planning. No listed amount is confirmed spent.</x:v>
+        <x:v>Historical estimates; use Launch Budget for current planning. Maryland LLC filing reported September 8, 2026; exact filing date and actual invoice amount unverified.</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -15503,10 +15507,8 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="41" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">LLC Formation (state TBD)</x:t>
-        </x:is>
+      <x:c r="A10" s="41" t="str">
+        <x:v>LLC formation — Maryland / Northwest</x:v>
       </x:c>
       <x:c r="B10" s="21" t="s">
         <x:v>478</x:v>
@@ -15521,13 +15523,11 @@
       <x:c r="F10" s="21" t="s">
         <x:v>470</x:v>
       </x:c>
-      <x:c r="G10" s="24" t="s">
-        <x:v>471</x:v>
-      </x:c>
-      <x:c r="H10" s="43" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Wyoming is a candidate for privacy/tax evaluation. Confirm state, registered agent, foreign qualification, and total cost with an attorney and CPA before filing.</x:t>
-        </x:is>
+      <x:c r="G10" s="24" t="str">
+        <x:v>Filed</x:v>
+      </x:c>
+      <x:c r="H10" s="43" t="str">
+        <x:v>Founder reports Kiban Digital Holdings LLC filed, awaiting Maryland approval. September 8 is the report date; filing date and payment amount unverified. D10 is historical, not the Northwest price.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -18282,7 +18282,7 @@
       </x:c>
       <x:c r="H8" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A8,'Delivery Tracker'!$H$4:$H$400,"In Progress")</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="I8" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A8,'Delivery Tracker'!$H$4:$H$400,"In Review")</x:f>
@@ -18294,10 +18294,10 @@
       </x:c>
       <x:c r="K8" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A8,'Delivery Tracker'!$H$4:$H$400,"Not Started")</x:f>
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="L8" s="111" t="str">
-        <x:v>Slices 1–3 are published, including PR #15. The private router remains dormant. Founder business definition is the next active task.</x:v>
+        <x:v>Slices 1–4 have published source; operations remain dormant. Founder reports Maryland LLC filed and CCBill inquiry sent. Await approval/response; review what arrives before another founder task.</x:v>
       </x:c>
       <x:c r="M8" s="111" t="str">
         <x:v>Resolve business/legal/provider prerequisites in sequence. G1–G12 apply to operations activation, not all synthetic local product work.</x:v>
@@ -18696,7 +18696,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="L15" s="111" t="str">
-        <x:v>Slice 3 is published in PR #15. Dormant private-operations foundation remains; further work is parked during founder business definition.</x:v>
+        <x:v>Dormant operations foundation has published source. Further operations work stays parked while Maryland approval and CCBill sales response are pending.</x:v>
       </x:c>
       <x:c r="M15" s="111" t="str">
         <x:v>Evaluate provider, restricted hosting, MFA/recovery, session, permission, audit and deployment controls when activating real operations.</x:v>
@@ -18962,7 +18962,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f8bb2389d85457d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f70c7d9d6084912"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19857,18 +19857,18 @@
         <x:v>Founder + provider response</x:v>
       </x:c>
       <x:c r="M18" s="111" t="str">
-        <x:v>Confirm dependencies and owner, then define the first deliverable.</x:v>
+        <x:v>Review the CCBill sales response for account-specific compliance requirements when received; assemble requested evidence in sequence afterward.</x:v>
       </x:c>
       <x:c r="N18" s="112"/>
       <x:c r="O18" s="111" t="str"/>
       <x:c r="P18" s="112" t="n">
-        <x:v>46250.666666666664</x:v>
+        <x:v>46273.666666666664</x:v>
       </x:c>
       <x:c r="Q18" s="111" t="str">
         <x:v>Document policies/controls required by CCBill and Epoch for merchant onboarding.</x:v>
       </x:c>
       <x:c r="R18" s="111" t="str">
-        <x:v>CCBill/Epoch applications have not started. Assemble the compliance package in parallel with product development.</x:v>
+        <x:v>Founder reports preliminary inquiry sent to CCBill sales. No response, formal merchant application or approval evidenced. Epoch may follow later. Await response before choosing another founder task.</x:v>
       </x:c>
       <x:c r="S18" s="111" t="str">
         <x:v>Preserved Master Tracker row 20; legacy status: 📋 Not Started</x:v>
@@ -20117,21 +20117,21 @@
         <x:v>Founder</x:v>
       </x:c>
       <x:c r="L23" s="111" t="str">
-        <x:v>Counsel / founder decision</x:v>
+        <x:v>Northwest / founder records</x:v>
       </x:c>
       <x:c r="M23" s="111" t="str">
-        <x:v>Close the remaining gap: Entity not filed.</x:v>
+        <x:v>Review the approved filing and published address details when Northwest supplies them; actual state approval remains pending.</x:v>
       </x:c>
       <x:c r="N23" s="112"/>
       <x:c r="O23" s="111" t="str"/>
       <x:c r="P23" s="112" t="n">
-        <x:v>46250.666666666664</x:v>
+        <x:v>46273.666666666664</x:v>
       </x:c>
       <x:c r="Q23" s="111" t="str">
         <x:v>Manage privacy concerns — MD biz records may expose personal identity linked to NSFW platform.</x:v>
       </x:c>
       <x:c r="R23" s="111" t="str">
-        <x:v>Entity not filed. Evaluate Wyoming and other privacy/no-individual-income-tax candidates with an attorney and CPA; account for foreign qualification where the founder operates.</x:v>
+        <x:v>Founder reports Kiban Digital Holdings LLC filed in Maryland through Northwest, awaiting approval. Final published address/privacy details remain unverified. State-comparison task is superseded.</x:v>
       </x:c>
       <x:c r="S23" s="111" t="str">
         <x:v>Preserved Master Tracker row 25; legacy status: 🔄 In Progress</x:v>
@@ -20999,7 +20999,7 @@
       </x:c>
       <x:c r="L40" s="111" t="str"/>
       <x:c r="M40" s="111" t="str">
-        <x:v>Define founding creator tag and fees-only offer with duration, eligibility and necessary fees before publication.</x:v>
+        <x:v>Define founder badge and a fee that recovers attributable costs without profit on founding creator sales. Duration, covered costs and no-loss economics need validation.</x:v>
       </x:c>
       <x:c r="N40" s="112"/>
       <x:c r="O40" s="111" t="str"/>
@@ -21010,7 +21010,7 @@
         <x:v>Define badge visuals, eligibility window (first N users or date window), locked-in fee reduction for Founding Creators, badge display on profiles and posts.</x:v>
       </x:c>
       <x:c r="R40" s="111" t="str">
-        <x:v>September 6, 2026: approximately500 creators is an acquisition target; Plus top100 leaderboard rewards are provisional. No public price/benefit promise yet.</x:v>
+        <x:v>Founder answers reviewed September 6, 2026: processing-fees-only superseded. Two contacts may recruit 50–100 prospects, not commitments. Longer target ~500; Plus/top 100 rewards remain provisional.</x:v>
       </x:c>
       <x:c r="S40" s="111" t="str">
         <x:v>Preserved Master Tracker row 43; legacy status: 📋 Not Started</x:v>
@@ -26426,10 +26426,10 @@
         <x:v>Legal &amp; compliance</x:v>
       </x:c>
       <x:c r="G145" s="111" t="str">
-        <x:v>Choose LLC state and privacy structure</x:v>
+        <x:v>Complete Maryland LLC formation</x:v>
       </x:c>
       <x:c r="H145" s="111" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="I145" s="111" t="str">
         <x:v>N/A</x:v>
@@ -26441,21 +26441,21 @@
         <x:v>Founder</x:v>
       </x:c>
       <x:c r="L145" s="111" t="str">
-        <x:v>Counsel / founder decision</x:v>
+        <x:v>Northwest / state approval</x:v>
       </x:c>
       <x:c r="M145" s="111" t="str">
-        <x:v>Confirm dependencies and owner, then define the first deliverable.</x:v>
+        <x:v>Await Maryland approval and approved documents. Filing is reported complete; exact filing date/ID, EIN, bank setup and actual invoice remain unverified.</x:v>
       </x:c>
       <x:c r="N145" s="112"/>
       <x:c r="O145" s="111" t="str"/>
       <x:c r="P145" s="112" t="n">
-        <x:v>46250.666666666664</x:v>
+        <x:v>46273.666666666664</x:v>
       </x:c>
       <x:c r="Q145" s="111" t="str">
-        <x:v>Compare Wyoming and other candidates with an adult-platform attorney and CPA; include registered agent, taxes, and foreign qualification.</x:v>
+        <x:v>Maryland LLC selected and filing reported by founder for Kiban Digital Holdings LLC through Northwest. Record approved filing and address details once returned.</x:v>
       </x:c>
       <x:c r="R145" s="111" t="str">
-        <x:v>No entity filed. A no-income-tax state does not by itself remove taxes or disclosure duties elsewhere.</x:v>
+        <x:v>Founder reported filing complete September 8, 2026; this is the report date, not a verified filing date. State approval pending. Filing ID and actual cost were not supplied.</x:v>
       </x:c>
       <x:c r="S145" s="111" t="str">
         <x:v>Preserved Master Tracker row 158; legacy status: 📋 Not Started</x:v>
@@ -27527,7 +27527,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79e8f6906de846af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc07a6951aab4717"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add Your Activity preview to phase 8
Move LEG-MT-080 into P08 and add protected member activity navigation, categorized sample history, search and month filters. Update the tracker, roadmap and handoff while retaining the pending account-history integration status.
</commit_message>
<xml_diff>
--- a/docs/product/Pumdoki_MasterTracker_V4.xlsx
+++ b/docs/product/Pumdoki_MasterTracker_V4.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re81aaddfa62f47b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="Rb5047abd3826488d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="R005d9f5f39f94900"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="Recd0c28599924730"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="R39c9842b214f462a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legacy Overview 2026-08-16" sheetId="6" r:id="Refdec6ae1cc1424c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="7" r:id="R8a341beb143b467c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Roadmap" sheetId="8" r:id="R760da7d95eb34f00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Tracker" sheetId="9" r:id="R322ee4ad41984bca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Blocker Queue" sheetId="10" r:id="R7ce6841af0e74069"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Log" sheetId="11" r:id="R445718308a854512"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Register" sheetId="12" r:id="R4e090ff29e2949a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Budget" sheetId="13" r:id="Rb6b02667adec4c3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R716f6b96a1924d94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Tracker" sheetId="2" r:id="R93dcd7e29dec4b75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" r:id="Rd0a8e2b0220d4ba5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes &amp; Assumptions" sheetId="4" r:id="R3eac5e89d79e4665"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💸 Expense Tracker" sheetId="5" r:id="Rba6512b08e9045d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legacy Overview 2026-08-16" sheetId="6" r:id="Rd21724ac9677451b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="7" r:id="Ra8f00a8c14254370"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Roadmap" sheetId="8" r:id="R48e6850903f243f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery Tracker" sheetId="9" r:id="R33358fc467cd41e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review &amp; Blocker Queue" sheetId="10" r:id="R3c9b8cfc375648e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Log" sheetId="11" r:id="R508e271d11dd4542"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Register" sheetId="12" r:id="Re0e57af217b94f6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Budget" sheetId="13" r:id="R097f08b44fd9486a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -580,9 +580,6 @@
     <x:t xml:space="preserve">Build 'Your Activity' page</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Nice-to-have post-launch. Defer if time is tight.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Improve Create Post ('Moments') modal</x:t>
   </x:si>
   <x:si>
@@ -1133,15 +1130,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Web-first; mobile later.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">'Your Activity' page</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">UX</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Nice-to-have. Build post-launch if time is tight during MVP push.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">TikTok paid creator promotions</x:t>
@@ -1742,7 +1730,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="23">
+  <x:fills count="24">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1852,6 +1840,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFC7CE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -1990,7 +1983,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="220">
+  <x:cellXfs count="221">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -2641,6 +2634,9 @@
     <x:xf numFmtId="0" fontId="30" fillId="22" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="23" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -3026,7 +3022,7 @@
         <x:color rgb="FF246B3B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF3E4"/>
         </x:patternFill>
       </x:fill>
@@ -3037,7 +3033,7 @@
         <x:color rgb="FF805E00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1C9"/>
         </x:patternFill>
       </x:fill>
@@ -3048,7 +3044,7 @@
         <x:color rgb="FF245B84"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDEBFA"/>
         </x:patternFill>
       </x:fill>
@@ -3059,7 +3055,7 @@
         <x:color rgb="FF8A2432"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF9D7DC"/>
         </x:patternFill>
       </x:fill>
@@ -3070,7 +3066,7 @@
         <x:color rgb="FF5D535C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFECE8EC"/>
         </x:patternFill>
       </x:fill>
@@ -3081,7 +3077,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -3092,7 +3088,7 @@
         <x:color rgb="FF246B3B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF3E4"/>
         </x:patternFill>
       </x:fill>
@@ -3103,7 +3099,7 @@
         <x:color rgb="FF805E00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1C9"/>
         </x:patternFill>
       </x:fill>
@@ -3114,7 +3110,7 @@
         <x:color rgb="FF245B84"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDEBFA"/>
         </x:patternFill>
       </x:fill>
@@ -3125,7 +3121,7 @@
         <x:color rgb="FF8A2432"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF9D7DC"/>
         </x:patternFill>
       </x:fill>
@@ -3136,7 +3132,7 @@
         <x:color rgb="FF5D535C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFECE8EC"/>
         </x:patternFill>
       </x:fill>
@@ -3147,7 +3143,7 @@
         <x:color rgb="FF3D1A3E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFAE1EC"/>
         </x:patternFill>
       </x:fill>
@@ -3158,7 +3154,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -3169,7 +3165,7 @@
         <x:color rgb="FF246B3B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF3E4"/>
         </x:patternFill>
       </x:fill>
@@ -3180,7 +3176,7 @@
         <x:color rgb="FF805E00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1C9"/>
         </x:patternFill>
       </x:fill>
@@ -3191,7 +3187,7 @@
         <x:color rgb="FF245B84"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDEBFA"/>
         </x:patternFill>
       </x:fill>
@@ -3202,7 +3198,7 @@
         <x:color rgb="FF8A2432"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF9D7DC"/>
         </x:patternFill>
       </x:fill>
@@ -3213,7 +3209,7 @@
         <x:color rgb="FF5D535C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFECE8EC"/>
         </x:patternFill>
       </x:fill>
@@ -3224,7 +3220,7 @@
         <x:color rgb="FF3D1A3E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFAE1EC"/>
         </x:patternFill>
       </x:fill>
@@ -3235,7 +3231,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -3246,7 +3242,7 @@
         <x:color rgb="FF246B3B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF3E4"/>
         </x:patternFill>
       </x:fill>
@@ -3257,7 +3253,7 @@
         <x:color rgb="FF805E00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1C9"/>
         </x:patternFill>
       </x:fill>
@@ -3268,7 +3264,7 @@
         <x:color rgb="FF245B84"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDEBFA"/>
         </x:patternFill>
       </x:fill>
@@ -3279,7 +3275,7 @@
         <x:color rgb="FF8A2432"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF9D7DC"/>
         </x:patternFill>
       </x:fill>
@@ -3290,7 +3286,7 @@
         <x:color rgb="FF5D535C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFECE8EC"/>
         </x:patternFill>
       </x:fill>
@@ -3301,7 +3297,7 @@
         <x:color rgb="FF3D1A3E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFAE1EC"/>
         </x:patternFill>
       </x:fill>
@@ -3312,7 +3308,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -3323,7 +3319,7 @@
         <x:color rgb="FF246B3B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF3E4"/>
         </x:patternFill>
       </x:fill>
@@ -3334,7 +3330,7 @@
         <x:color rgb="FF805E00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1C9"/>
         </x:patternFill>
       </x:fill>
@@ -3345,7 +3341,7 @@
         <x:color rgb="FF245B84"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDEBFA"/>
         </x:patternFill>
       </x:fill>
@@ -3356,7 +3352,7 @@
         <x:color rgb="FF8A2432"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF9D7DC"/>
         </x:patternFill>
       </x:fill>
@@ -3367,7 +3363,7 @@
         <x:color rgb="FF5D535C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFECE8EC"/>
         </x:patternFill>
       </x:fill>
@@ -3378,7 +3374,7 @@
         <x:color rgb="FF3D1A3E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFAE1EC"/>
         </x:patternFill>
       </x:fill>
@@ -3389,7 +3385,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -3400,7 +3396,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -3411,7 +3407,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -3943,7 +3939,7 @@
       <x:c r="D13" s="151"/>
       <x:c r="E13" s="150" t="n">
         <x:f>COUNTIF('Delivery Tracker'!$H$4:$H$400,"In Progress")</x:f>
-        <x:v>52</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="F13" s="151"/>
       <x:c r="G13" s="150" t="n">
@@ -3958,7 +3954,7 @@
       <x:c r="J13" s="151"/>
       <x:c r="K13" s="150" t="n">
         <x:f>COUNTIF('Delivery Tracker'!$H$4:$H$400,"Not Started")</x:f>
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="L13" s="151"/>
       <x:c r="M13" s="158" t="n">
@@ -4536,15 +4532,15 @@
       </x:c>
       <x:c r="F26" s="111" t="n">
         <x:f>'Phase Roadmap'!F12</x:f>
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G26" s="119" t="n">
         <x:f>'Phase Roadmap'!G12</x:f>
-        <x:v>0.4444444444444444</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="H26" s="111" t="n">
         <x:f>'Phase Roadmap'!H12</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="I26" s="111" t="n">
         <x:f>'Phase Roadmap'!I12</x:f>
@@ -4560,11 +4556,11 @@
       </x:c>
       <x:c r="L26" s="111" t="str">
         <x:f>'Phase Roadmap'!L12</x:f>
-        <x:v>Connect discovery, Store and feed remain launch scope. Connect means online, price and language filters.</x:v>
+        <x:v>Feed, Store and Connect remain launch scope (online/price/language discovery). Your Activity /activity UI is an explicit example-data preview; real member history remains pending.</x:v>
       </x:c>
       <x:c r="M26" s="111" t="str">
         <x:f>'Phase Roadmap'!M12</x:f>
-        <x:v>Integrate content and access controls. Define service/order and beta payment rules with the relevant slice.</x:v>
+        <x:v>Integrate content/access, service/order and beta payment rules. Connect Your Activity to authenticated P05/P06/P07 data.</x:v>
       </x:c>
       <x:c r="N26" s="111" t="str">
         <x:f>'Phase Roadmap'!O12</x:f>
@@ -6367,7 +6363,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46f208786e734731"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb3347981fce4ac2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7489,7 +7485,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe125cfc69b24b7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3a41e2639444792"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8344,7 +8340,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf4d4d30ca3e45c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a6f89c65da04024"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10338,63 +10334,63 @@
         <x:v>185</x:v>
       </x:c>
       <x:c r="B80" s="17" t="str">
-        <x:v>Member activity history: posts liked, content purchased, subscriptions and payment history. Lower priority.</x:v>
-      </x:c>
-      <x:c r="C80" s="24" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="D80" s="19" t="s">
-        <x:v>186</x:v>
+        <x:v>P08 member history: liked posts, purchases, subscriptions and payment history. UI preview first; account-backed events follow.</x:v>
+      </x:c>
+      <x:c r="C80" s="220" t="str">
+        <x:v>🔄 In Progress</x:v>
+      </x:c>
+      <x:c r="D80" s="19" t="str">
+        <x:v>Example-data /activity UI with search/filters and sidebar/header links. Real account API and persistence pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="15.75" customHeight="1">
       <x:c r="A81" s="20" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="B81" s="21" t="s">
         <x:v>187</x:v>
-      </x:c>
-      <x:c r="B81" s="21" t="s">
-        <x:v>188</x:v>
       </x:c>
       <x:c r="C81" s="18" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="D81" s="22" t="s">
-        <x:v>189</x:v>
+        <x:v>188</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="15.75" customHeight="1">
       <x:c r="A82" s="16" t="s">
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="B82" s="17" t="s">
         <x:v>190</x:v>
-      </x:c>
-      <x:c r="B82" s="17" t="s">
-        <x:v>191</x:v>
       </x:c>
       <x:c r="C82" s="18" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="D82" s="19" t="s">
-        <x:v>192</x:v>
+        <x:v>191</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="15.75" customHeight="1">
       <x:c r="A83" s="20" t="s">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="B83" s="21" t="s">
         <x:v>193</x:v>
-      </x:c>
-      <x:c r="B83" s="21" t="s">
-        <x:v>194</x:v>
       </x:c>
       <x:c r="C83" s="18" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="D83" s="22" t="s">
-        <x:v>195</x:v>
+        <x:v>194</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="30.75" customHeight="1">
       <x:c r="A84" s="16" t="s">
+        <x:v>195</x:v>
+      </x:c>
+      <x:c r="B84" s="17" t="s">
         <x:v>196</x:v>
-      </x:c>
-      <x:c r="B84" s="17" t="s">
-        <x:v>197</x:v>
       </x:c>
       <x:c r="C84" s="23" t="inlineStr">
         <x:is>
@@ -10409,21 +10405,21 @@
     </x:row>
     <x:row r="85" ht="18.75" customHeight="1">
       <x:c r="A85" s="25" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="B85" s="26" t="s">
         <x:v>198</x:v>
-      </x:c>
-      <x:c r="B85" s="26" t="s">
-        <x:v>199</x:v>
       </x:c>
       <x:c r="C85" s="18" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="D85" s="27" t="s">
-        <x:v>200</x:v>
+        <x:v>199</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="15.75" customHeight="1">
       <x:c r="A86" s="15" t="s">
-        <x:v>201</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="B86" s="2"/>
       <x:c r="C86" s="2"/>
@@ -10431,91 +10427,91 @@
     </x:row>
     <x:row r="87" ht="15.75" customHeight="1">
       <x:c r="A87" s="16" t="s">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="B87" s="17" t="s">
         <x:v>202</x:v>
-      </x:c>
-      <x:c r="B87" s="17" t="s">
-        <x:v>203</x:v>
       </x:c>
       <x:c r="C87" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D87" s="19" t="s">
-        <x:v>204</x:v>
+        <x:v>203</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="15.75" customHeight="1">
       <x:c r="A88" s="20" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="B88" s="21" t="s">
         <x:v>205</x:v>
-      </x:c>
-      <x:c r="B88" s="21" t="s">
-        <x:v>206</x:v>
       </x:c>
       <x:c r="C88" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D88" s="22" t="s">
-        <x:v>207</x:v>
+        <x:v>206</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="15.75" customHeight="1">
       <x:c r="A89" s="16" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="B89" s="17" t="s">
         <x:v>208</x:v>
-      </x:c>
-      <x:c r="B89" s="17" t="s">
-        <x:v>209</x:v>
       </x:c>
       <x:c r="C89" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D89" s="19" t="s">
-        <x:v>210</x:v>
+        <x:v>209</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="15.75" customHeight="1">
       <x:c r="A90" s="20" t="s">
+        <x:v>210</x:v>
+      </x:c>
+      <x:c r="B90" s="21" t="s">
         <x:v>211</x:v>
-      </x:c>
-      <x:c r="B90" s="21" t="s">
-        <x:v>212</x:v>
       </x:c>
       <x:c r="C90" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D90" s="22" t="s">
-        <x:v>213</x:v>
+        <x:v>212</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="15.75" customHeight="1">
       <x:c r="A91" s="16" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="B91" s="17" t="s">
         <x:v>214</x:v>
-      </x:c>
-      <x:c r="B91" s="17" t="s">
-        <x:v>215</x:v>
       </x:c>
       <x:c r="C91" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D91" s="19" t="s">
-        <x:v>216</x:v>
+        <x:v>215</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="27.75" customHeight="1">
       <x:c r="A92" s="28" t="s">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="B92" s="29" t="s">
         <x:v>217</x:v>
-      </x:c>
-      <x:c r="B92" s="29" t="s">
-        <x:v>218</x:v>
       </x:c>
       <x:c r="C92" s="30" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D92" s="31" t="s">
-        <x:v>219</x:v>
+        <x:v>218</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="15.75" customHeight="1">
       <x:c r="A93" s="15" t="s">
-        <x:v>220</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="B93" s="2"/>
       <x:c r="C93" s="2"/>
@@ -10523,10 +10519,10 @@
     </x:row>
     <x:row r="94" ht="15.75" customHeight="1">
       <x:c r="A94" s="32" t="s">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="B94" s="33" t="s">
         <x:v>221</x:v>
-      </x:c>
-      <x:c r="B94" s="33" t="s">
-        <x:v>222</x:v>
       </x:c>
       <x:c r="C94" s="217" t="str">
         <x:v>🔄 In Progress</x:v>
@@ -10537,10 +10533,10 @@
     </x:row>
     <x:row r="95" ht="15.75" customHeight="1">
       <x:c r="A95" s="20" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="B95" s="21" t="s">
         <x:v>223</x:v>
-      </x:c>
-      <x:c r="B95" s="21" t="s">
-        <x:v>224</x:v>
       </x:c>
       <x:c r="C95" s="24" t="inlineStr">
         <x:is>
@@ -10553,10 +10549,10 @@
     </x:row>
     <x:row r="96" ht="15.75" customHeight="1">
       <x:c r="A96" s="16" t="s">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="B96" s="17" t="s">
         <x:v>225</x:v>
-      </x:c>
-      <x:c r="B96" s="17" t="s">
-        <x:v>226</x:v>
       </x:c>
       <x:c r="C96" s="24" t="s">
         <x:v>21</x:v>
@@ -10567,10 +10563,10 @@
     </x:row>
     <x:row r="97" ht="15.75" customHeight="1">
       <x:c r="A97" s="20" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="B97" s="21" t="s">
         <x:v>227</x:v>
-      </x:c>
-      <x:c r="B97" s="21" t="s">
-        <x:v>228</x:v>
       </x:c>
       <x:c r="C97" s="24" t="s">
         <x:v>21</x:v>
@@ -10581,44 +10577,44 @@
     </x:row>
     <x:row r="98" ht="15.75" customHeight="1">
       <x:c r="A98" s="16" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="B98" s="17" t="s">
         <x:v>229</x:v>
-      </x:c>
-      <x:c r="B98" s="17" t="s">
-        <x:v>230</x:v>
       </x:c>
       <x:c r="C98" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D98" s="19" t="s">
-        <x:v>231</x:v>
+        <x:v>230</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="15.75" customHeight="1">
       <x:c r="A99" s="20" t="s">
+        <x:v>231</x:v>
+      </x:c>
+      <x:c r="B99" s="21" t="s">
         <x:v>232</x:v>
-      </x:c>
-      <x:c r="B99" s="21" t="s">
-        <x:v>233</x:v>
       </x:c>
       <x:c r="C99" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D99" s="22" t="s">
-        <x:v>234</x:v>
+        <x:v>233</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="15.75" customHeight="1">
       <x:c r="A100" s="16" t="s">
+        <x:v>234</x:v>
+      </x:c>
+      <x:c r="B100" s="17" t="s">
         <x:v>235</x:v>
-      </x:c>
-      <x:c r="B100" s="17" t="s">
-        <x:v>236</x:v>
       </x:c>
       <x:c r="C100" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D100" s="19" t="s">
-        <x:v>237</x:v>
+        <x:v>236</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="15.75" customHeight="1">
@@ -10629,10 +10625,10 @@
     </x:row>
     <x:row r="102" ht="15.75" customHeight="1">
       <x:c r="A102" s="16" t="s">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="B102" s="17" t="s">
         <x:v>238</x:v>
-      </x:c>
-      <x:c r="B102" s="17" t="s">
-        <x:v>239</x:v>
       </x:c>
       <x:c r="C102" s="24" t="s">
         <x:v>21</x:v>
@@ -10645,10 +10641,10 @@
     </x:row>
     <x:row r="103" ht="15.75" customHeight="1">
       <x:c r="A103" s="20" t="s">
+        <x:v>239</x:v>
+      </x:c>
+      <x:c r="B103" s="21" t="s">
         <x:v>240</x:v>
-      </x:c>
-      <x:c r="B103" s="21" t="s">
-        <x:v>241</x:v>
       </x:c>
       <x:c r="C103" s="24" t="s">
         <x:v>21</x:v>
@@ -10659,21 +10655,21 @@
     </x:row>
     <x:row r="104" ht="27.75" customHeight="1">
       <x:c r="A104" s="36" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="B104" s="37" t="s">
         <x:v>242</x:v>
-      </x:c>
-      <x:c r="B104" s="37" t="s">
-        <x:v>243</x:v>
       </x:c>
       <x:c r="C104" s="30" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D104" s="38" t="s">
-        <x:v>244</x:v>
+        <x:v>243</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="15.75" customHeight="1">
       <x:c r="A105" s="15" t="s">
-        <x:v>245</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="B105" s="2"/>
       <x:c r="C105" s="2"/>
@@ -10695,38 +10691,38 @@
     </x:row>
     <x:row r="107" ht="15" hidden="0" customHeight="1">
       <x:c r="A107" s="20" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="B107" s="21" t="s">
         <x:v>246</x:v>
-      </x:c>
-      <x:c r="B107" s="21" t="s">
-        <x:v>247</x:v>
       </x:c>
       <x:c r="C107" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D107" s="22" t="s">
-        <x:v>248</x:v>
+        <x:v>247</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="15" hidden="0" customHeight="1">
       <x:c r="A108" s="16" t="s">
+        <x:v>248</x:v>
+      </x:c>
+      <x:c r="B108" s="17" t="s">
         <x:v>249</x:v>
-      </x:c>
-      <x:c r="B108" s="17" t="s">
-        <x:v>250</x:v>
       </x:c>
       <x:c r="C108" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D108" s="19" t="s">
-        <x:v>251</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="24" hidden="0" customHeight="1">
       <x:c r="A109" s="20" t="s">
+        <x:v>251</x:v>
+      </x:c>
+      <x:c r="B109" s="21" t="s">
         <x:v>252</x:v>
-      </x:c>
-      <x:c r="B109" s="21" t="s">
-        <x:v>253</x:v>
       </x:c>
       <x:c r="C109" s="24" t="str">
         <x:v>🔄 In Progress</x:v>
@@ -10737,38 +10733,38 @@
     </x:row>
     <x:row r="110" ht="15.75" customHeight="1">
       <x:c r="A110" s="16" t="s">
+        <x:v>253</x:v>
+      </x:c>
+      <x:c r="B110" s="17" t="s">
         <x:v>254</x:v>
-      </x:c>
-      <x:c r="B110" s="17" t="s">
-        <x:v>255</x:v>
       </x:c>
       <x:c r="C110" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D110" s="19" t="s">
-        <x:v>256</x:v>
+        <x:v>255</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="15.75" customHeight="1">
       <x:c r="A111" s="20" t="s">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="B111" s="21" t="s">
         <x:v>257</x:v>
-      </x:c>
-      <x:c r="B111" s="21" t="s">
-        <x:v>258</x:v>
       </x:c>
       <x:c r="C111" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D111" s="22" t="s">
-        <x:v>259</x:v>
+        <x:v>258</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="15.75" customHeight="1">
       <x:c r="A112" s="16" t="s">
+        <x:v>259</x:v>
+      </x:c>
+      <x:c r="B112" s="17" t="s">
         <x:v>260</x:v>
-      </x:c>
-      <x:c r="B112" s="17" t="s">
-        <x:v>261</x:v>
       </x:c>
       <x:c r="C112" s="24" t="s">
         <x:v>21</x:v>
@@ -10779,7 +10775,7 @@
     </x:row>
     <x:row r="113" ht="15.75" customHeight="1">
       <x:c r="A113" s="20" t="s">
-        <x:v>262</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="B113" s="21" t="str">
         <x:v>View verified processor chargeback events, calculate rates, apply confirmed account-specific alert thresholds and log authorized dispute responses.</x:v>
@@ -10799,52 +10795,52 @@
     </x:row>
     <x:row r="115" ht="15.75" customHeight="1">
       <x:c r="A115" s="20" t="s">
+        <x:v>262</x:v>
+      </x:c>
+      <x:c r="B115" s="21" t="s">
         <x:v>263</x:v>
-      </x:c>
-      <x:c r="B115" s="21" t="s">
-        <x:v>264</x:v>
       </x:c>
       <x:c r="C115" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D115" s="22" t="s">
-        <x:v>265</x:v>
+        <x:v>264</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="15.75" customHeight="1">
       <x:c r="A116" s="16" t="s">
+        <x:v>265</x:v>
+      </x:c>
+      <x:c r="B116" s="17" t="s">
         <x:v>266</x:v>
-      </x:c>
-      <x:c r="B116" s="17" t="s">
-        <x:v>267</x:v>
       </x:c>
       <x:c r="C116" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D116" s="19" t="s">
-        <x:v>268</x:v>
+        <x:v>267</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="15.75" customHeight="1">
       <x:c r="A117" s="20" t="s">
+        <x:v>268</x:v>
+      </x:c>
+      <x:c r="B117" s="21" t="s">
         <x:v>269</x:v>
-      </x:c>
-      <x:c r="B117" s="21" t="s">
-        <x:v>270</x:v>
       </x:c>
       <x:c r="C117" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D117" s="22" t="s">
-        <x:v>271</x:v>
+        <x:v>270</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="24" hidden="0" customHeight="1">
       <x:c r="A118" s="36" t="s">
+        <x:v>271</x:v>
+      </x:c>
+      <x:c r="B118" s="37" t="s">
         <x:v>272</x:v>
-      </x:c>
-      <x:c r="B118" s="37" t="s">
-        <x:v>273</x:v>
       </x:c>
       <x:c r="C118" s="30" t="s">
         <x:v>21</x:v>
@@ -10855,7 +10851,7 @@
     </x:row>
     <x:row r="119" ht="15.75" customHeight="1">
       <x:c r="A119" s="15" t="s">
-        <x:v>274</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="B119" s="2"/>
       <x:c r="C119" s="2"/>
@@ -10863,10 +10859,10 @@
     </x:row>
     <x:row r="120" ht="15.75" customHeight="1">
       <x:c r="A120" s="32" t="s">
+        <x:v>274</x:v>
+      </x:c>
+      <x:c r="B120" s="33" t="s">
         <x:v>275</x:v>
-      </x:c>
-      <x:c r="B120" s="33" t="s">
-        <x:v>276</x:v>
       </x:c>
       <x:c r="C120" s="39" t="s">
         <x:v>21</x:v>
@@ -10877,52 +10873,52 @@
     </x:row>
     <x:row r="121" ht="15.75" customHeight="1">
       <x:c r="A121" s="20" t="s">
+        <x:v>276</x:v>
+      </x:c>
+      <x:c r="B121" s="21" t="s">
         <x:v>277</x:v>
-      </x:c>
-      <x:c r="B121" s="21" t="s">
-        <x:v>278</x:v>
       </x:c>
       <x:c r="C121" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D121" s="22" t="s">
-        <x:v>279</x:v>
+        <x:v>278</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="15.75" customHeight="1">
       <x:c r="A122" s="16" t="s">
+        <x:v>279</x:v>
+      </x:c>
+      <x:c r="B122" s="17" t="s">
         <x:v>280</x:v>
-      </x:c>
-      <x:c r="B122" s="17" t="s">
-        <x:v>281</x:v>
       </x:c>
       <x:c r="C122" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D122" s="19" t="s">
-        <x:v>282</x:v>
+        <x:v>281</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="15.75" customHeight="1">
       <x:c r="A123" s="20" t="s">
+        <x:v>282</x:v>
+      </x:c>
+      <x:c r="B123" s="21" t="s">
         <x:v>283</x:v>
-      </x:c>
-      <x:c r="B123" s="21" t="s">
-        <x:v>284</x:v>
       </x:c>
       <x:c r="C123" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D123" s="22" t="s">
-        <x:v>285</x:v>
+        <x:v>284</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="24" hidden="0" customHeight="1">
       <x:c r="A124" s="36" t="s">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="B124" s="37" t="s">
         <x:v>286</x:v>
-      </x:c>
-      <x:c r="B124" s="37" t="s">
-        <x:v>287</x:v>
       </x:c>
       <x:c r="C124" s="30" t="str">
         <x:v>🔄 In Progress</x:v>
@@ -10933,7 +10929,7 @@
     </x:row>
     <x:row r="125" ht="15.75" customHeight="1">
       <x:c r="A125" s="15" t="s">
-        <x:v>288</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="B125" s="2"/>
       <x:c r="C125" s="2"/>
@@ -10941,105 +10937,105 @@
     </x:row>
     <x:row r="126" ht="15.75" customHeight="1">
       <x:c r="A126" s="32" t="s">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="B126" s="33" t="s">
         <x:v>289</x:v>
-      </x:c>
-      <x:c r="B126" s="33" t="s">
-        <x:v>290</x:v>
       </x:c>
       <x:c r="C126" s="39" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D126" s="35" t="s">
-        <x:v>291</x:v>
+        <x:v>290</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="15.75" customHeight="1">
       <x:c r="A127" s="20" t="s">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="B127" s="21" t="s">
         <x:v>292</x:v>
-      </x:c>
-      <x:c r="B127" s="21" t="s">
-        <x:v>293</x:v>
       </x:c>
       <x:c r="C127" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D127" s="22" t="s">
-        <x:v>294</x:v>
+        <x:v>293</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="15.75" customHeight="1">
       <x:c r="A128" s="16" t="s">
+        <x:v>294</x:v>
+      </x:c>
+      <x:c r="B128" s="17" t="s">
         <x:v>295</x:v>
-      </x:c>
-      <x:c r="B128" s="17" t="s">
-        <x:v>296</x:v>
       </x:c>
       <x:c r="C128" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D128" s="19" t="s">
-        <x:v>297</x:v>
+        <x:v>296</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="15.75" customHeight="1">
       <x:c r="A129" s="20" t="s">
+        <x:v>297</x:v>
+      </x:c>
+      <x:c r="B129" s="21" t="s">
         <x:v>298</x:v>
-      </x:c>
-      <x:c r="B129" s="21" t="s">
-        <x:v>299</x:v>
       </x:c>
       <x:c r="C129" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D129" s="22" t="s">
-        <x:v>300</x:v>
+        <x:v>299</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="15.75" customHeight="1">
       <x:c r="A130" s="16" t="s">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="B130" s="17" t="s">
         <x:v>301</x:v>
-      </x:c>
-      <x:c r="B130" s="17" t="s">
-        <x:v>302</x:v>
       </x:c>
       <x:c r="C130" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D130" s="19" t="s">
-        <x:v>303</x:v>
+        <x:v>302</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="15" customHeight="1">
       <x:c r="A131" s="20" t="s">
+        <x:v>303</x:v>
+      </x:c>
+      <x:c r="B131" s="21" t="s">
         <x:v>304</x:v>
-      </x:c>
-      <x:c r="B131" s="21" t="s">
-        <x:v>305</x:v>
       </x:c>
       <x:c r="C131" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D131" s="22" t="s">
-        <x:v>306</x:v>
+        <x:v>305</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="15.75" customHeight="1">
       <x:c r="A132" s="40" t="s">
+        <x:v>306</x:v>
+      </x:c>
+      <x:c r="B132" s="41" t="s">
         <x:v>307</x:v>
-      </x:c>
-      <x:c r="B132" s="41" t="s">
-        <x:v>308</x:v>
       </x:c>
       <x:c r="C132" s="42" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="D132" s="43" t="s">
-        <x:v>303</x:v>
+        <x:v>302</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="15.75" customHeight="1">
       <x:c r="A133" s="15" t="s">
-        <x:v>309</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="B133" s="2"/>
       <x:c r="C133" s="2"/>
@@ -11047,10 +11043,10 @@
     </x:row>
     <x:row r="134" ht="24" hidden="0" customHeight="1">
       <x:c r="A134" s="32" t="s">
+        <x:v>309</x:v>
+      </x:c>
+      <x:c r="B134" s="33" t="s">
         <x:v>310</x:v>
-      </x:c>
-      <x:c r="B134" s="33" t="s">
-        <x:v>311</x:v>
       </x:c>
       <x:c r="C134" s="44" t="s">
         <x:v>26</x:v>
@@ -11061,52 +11057,52 @@
     </x:row>
     <x:row r="135" ht="15.75" customHeight="1">
       <x:c r="A135" s="20" t="s">
+        <x:v>311</x:v>
+      </x:c>
+      <x:c r="B135" s="21" t="s">
         <x:v>312</x:v>
-      </x:c>
-      <x:c r="B135" s="21" t="s">
-        <x:v>313</x:v>
       </x:c>
       <x:c r="C135" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D135" s="22" t="s">
-        <x:v>314</x:v>
+        <x:v>313</x:v>
       </x:c>
     </x:row>
     <x:row r="136" ht="15.75" customHeight="1">
       <x:c r="A136" s="16" t="s">
+        <x:v>314</x:v>
+      </x:c>
+      <x:c r="B136" s="17" t="s">
         <x:v>315</x:v>
-      </x:c>
-      <x:c r="B136" s="17" t="s">
-        <x:v>316</x:v>
       </x:c>
       <x:c r="C136" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D136" s="19" t="s">
-        <x:v>317</x:v>
+        <x:v>316</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="15.75" customHeight="1">
       <x:c r="A137" s="20" t="s">
+        <x:v>317</x:v>
+      </x:c>
+      <x:c r="B137" s="21" t="s">
         <x:v>318</x:v>
-      </x:c>
-      <x:c r="B137" s="21" t="s">
-        <x:v>319</x:v>
       </x:c>
       <x:c r="C137" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D137" s="22" t="s">
-        <x:v>303</x:v>
+        <x:v>302</x:v>
       </x:c>
     </x:row>
     <x:row r="138" ht="15.75" customHeight="1">
       <x:c r="A138" s="16" t="s">
+        <x:v>319</x:v>
+      </x:c>
+      <x:c r="B138" s="17" t="s">
         <x:v>320</x:v>
-      </x:c>
-      <x:c r="B138" s="17" t="s">
-        <x:v>321</x:v>
       </x:c>
       <x:c r="C138" s="24" t="s">
         <x:v>21</x:v>
@@ -11117,44 +11113,44 @@
     </x:row>
     <x:row r="139" ht="15.75" customHeight="1">
       <x:c r="A139" s="20" t="s">
+        <x:v>321</x:v>
+      </x:c>
+      <x:c r="B139" s="21" t="s">
         <x:v>322</x:v>
-      </x:c>
-      <x:c r="B139" s="21" t="s">
-        <x:v>323</x:v>
       </x:c>
       <x:c r="C139" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D139" s="22" t="s">
-        <x:v>324</x:v>
+        <x:v>323</x:v>
       </x:c>
     </x:row>
     <x:row r="140" ht="15.75" customHeight="1">
       <x:c r="A140" s="16" t="s">
+        <x:v>324</x:v>
+      </x:c>
+      <x:c r="B140" s="17" t="s">
         <x:v>325</x:v>
-      </x:c>
-      <x:c r="B140" s="17" t="s">
-        <x:v>326</x:v>
       </x:c>
       <x:c r="C140" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D140" s="19" t="s">
-        <x:v>327</x:v>
+        <x:v>326</x:v>
       </x:c>
     </x:row>
     <x:row r="141" ht="15.75" customHeight="1">
       <x:c r="A141" s="20" t="s">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="B141" s="21" t="s">
         <x:v>328</x:v>
-      </x:c>
-      <x:c r="B141" s="21" t="s">
-        <x:v>329</x:v>
       </x:c>
       <x:c r="C141" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="D141" s="22" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
     </x:row>
     <x:row r="142" ht="27.75" customHeight="1">
@@ -12468,50 +12464,50 @@
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
       <x:c r="A1" s="14" t="s">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="B1" s="14" t="s">
         <x:v>331</x:v>
       </x:c>
-      <x:c r="B1" s="14" t="s">
+      <x:c r="C1" s="14" t="s">
         <x:v>332</x:v>
       </x:c>
-      <x:c r="C1" s="14" t="s">
+      <x:c r="D1" s="14" t="s">
         <x:v>333</x:v>
-      </x:c>
-      <x:c r="D1" s="14" t="s">
-        <x:v>334</x:v>
       </x:c>
       <x:c r="E1" s="14" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="F1" s="14" t="s">
-        <x:v>335</x:v>
+        <x:v>334</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="20" t="s">
+        <x:v>335</x:v>
+      </x:c>
+      <x:c r="B2" s="21" t="s">
         <x:v>336</x:v>
       </x:c>
-      <x:c r="B2" s="21" t="s">
+      <x:c r="C2" s="21" t="s">
         <x:v>337</x:v>
       </x:c>
-      <x:c r="C2" s="21" t="s">
+      <x:c r="D2" s="21" t="s">
         <x:v>338</x:v>
-      </x:c>
-      <x:c r="D2" s="21" t="s">
-        <x:v>339</x:v>
       </x:c>
       <x:c r="E2" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="F2" s="21" t="s">
-        <x:v>340</x:v>
+        <x:v>339</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="16" t="s">
-        <x:v>341</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="B3" s="17" t="s">
-        <x:v>337</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="C3" s="21" t="inlineStr">
         <x:is>
@@ -12519,7 +12515,7 @@
         </x:is>
       </x:c>
       <x:c r="D3" s="17" t="s">
-        <x:v>339</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="E3" s="24" t="s">
         <x:v>21</x:v>
@@ -12532,10 +12528,10 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="20" t="s">
+        <x:v>341</x:v>
+      </x:c>
+      <x:c r="B4" s="21" t="s">
         <x:v>342</x:v>
-      </x:c>
-      <x:c r="B4" s="21" t="s">
-        <x:v>343</x:v>
       </x:c>
       <x:c r="C4" s="21" t="inlineStr">
         <x:is>
@@ -12560,10 +12556,10 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="16" t="s">
-        <x:v>344</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="B5" s="17" t="s">
-        <x:v>343</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="C5" s="17" t="inlineStr">
         <x:is>
@@ -12588,42 +12584,42 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="20" t="s">
+        <x:v>344</x:v>
+      </x:c>
+      <x:c r="B6" s="21" t="s">
         <x:v>345</x:v>
       </x:c>
-      <x:c r="B6" s="21" t="s">
+      <x:c r="C6" s="21" t="s">
         <x:v>346</x:v>
       </x:c>
-      <x:c r="C6" s="21" t="s">
-        <x:v>347</x:v>
-      </x:c>
       <x:c r="D6" s="21" t="s">
-        <x:v>339</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="E6" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="F6" s="21" t="s">
-        <x:v>340</x:v>
+        <x:v>339</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="16" t="s">
+        <x:v>347</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="s">
         <x:v>348</x:v>
       </x:c>
-      <x:c r="B7" s="17" t="s">
+      <x:c r="C7" s="17" t="s">
         <x:v>349</x:v>
       </x:c>
-      <x:c r="C7" s="17" t="s">
+      <x:c r="D7" s="17" t="s">
         <x:v>350</x:v>
-      </x:c>
-      <x:c r="D7" s="17" t="s">
-        <x:v>351</x:v>
       </x:c>
       <x:c r="E7" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="F7" s="17" t="s">
-        <x:v>340</x:v>
+        <x:v>339</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -12631,27 +12627,27 @@
         <x:v>Multiple themes (beyond Sakura Kiss &amp; Midnight City)</x:v>
       </x:c>
       <x:c r="B8" s="21" t="s">
+        <x:v>351</x:v>
+      </x:c>
+      <x:c r="C8" s="21" t="s">
         <x:v>352</x:v>
       </x:c>
-      <x:c r="C8" s="21" t="s">
-        <x:v>353</x:v>
-      </x:c>
       <x:c r="D8" s="21" t="s">
-        <x:v>351</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="E8" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="F8" s="21" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="16" t="s">
-        <x:v>355</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="B9" s="17" t="s">
-        <x:v>337</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="C9" s="17" t="inlineStr">
         <x:is>
@@ -12676,162 +12672,150 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="20" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="B10" s="21" t="s">
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="C10" s="21" t="s">
         <x:v>356</x:v>
       </x:c>
-      <x:c r="B10" s="21" t="s">
-        <x:v>343</x:v>
-      </x:c>
-      <x:c r="C10" s="21" t="s">
-        <x:v>357</x:v>
-      </x:c>
       <x:c r="D10" s="21" t="s">
-        <x:v>339</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="E10" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="F10" s="21" t="s">
-        <x:v>358</x:v>
+        <x:v>357</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="16" t="s">
+        <x:v>358</x:v>
+      </x:c>
+      <x:c r="B11" s="17" t="s">
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="C11" s="17" t="s">
         <x:v>359</x:v>
       </x:c>
-      <x:c r="B11" s="17" t="s">
-        <x:v>343</x:v>
-      </x:c>
-      <x:c r="C11" s="17" t="s">
-        <x:v>360</x:v>
-      </x:c>
       <x:c r="D11" s="17" t="s">
-        <x:v>339</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="E11" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="F11" s="17" t="s">
-        <x:v>361</x:v>
+        <x:v>360</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="20" t="s">
+        <x:v>361</x:v>
+      </x:c>
+      <x:c r="B12" s="21" t="s">
         <x:v>362</x:v>
       </x:c>
-      <x:c r="B12" s="21" t="s">
+      <x:c r="C12" s="21" t="s">
         <x:v>363</x:v>
       </x:c>
-      <x:c r="C12" s="21" t="s">
-        <x:v>364</x:v>
-      </x:c>
       <x:c r="D12" s="21" t="s">
-        <x:v>339</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="E12" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="F12" s="21" t="s">
-        <x:v>365</x:v>
+        <x:v>364</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="16" t="s">
+        <x:v>365</x:v>
+      </x:c>
+      <x:c r="B13" s="17" t="s">
         <x:v>366</x:v>
       </x:c>
-      <x:c r="B13" s="17" t="s">
+      <x:c r="C13" s="17" t="s">
         <x:v>367</x:v>
       </x:c>
-      <x:c r="C13" s="17" t="s">
+      <x:c r="D13" s="17" t="s">
         <x:v>368</x:v>
-      </x:c>
-      <x:c r="D13" s="17" t="s">
-        <x:v>369</x:v>
       </x:c>
       <x:c r="E13" s="24" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="F13" s="17" t="s">
-        <x:v>370</x:v>
+        <x:v>369</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="20" t="s">
-        <x:v>371</x:v>
-      </x:c>
-      <x:c r="B14" s="21" t="s">
-        <x:v>372</x:v>
-      </x:c>
-      <x:c r="C14" s="21" t="str">
-        <x:v>Activity history for members: posts liked, content purchased and payment history.</x:v>
-      </x:c>
-      <x:c r="D14" s="21" t="s">
-        <x:v>351</x:v>
-      </x:c>
-      <x:c r="E14" s="24" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="F14" s="21" t="s">
-        <x:v>373</x:v>
-      </x:c>
+      <x:c r="A14" s="20"/>
+      <x:c r="B14" s="21"/>
+      <x:c r="C14" s="21"/>
+      <x:c r="D14" s="21"/>
+      <x:c r="E14" s="24"/>
+      <x:c r="F14" s="21"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="45" t="s">
-        <x:v>374</x:v>
+        <x:v>370</x:v>
       </x:c>
       <x:c r="B15" s="46" t="s">
-        <x:v>375</x:v>
+        <x:v>371</x:v>
       </x:c>
       <x:c r="C15" s="47" t="s">
-        <x:v>376</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="D15" s="46" t="s">
-        <x:v>339</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="E15" s="48" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="F15" s="47" t="s">
-        <x:v>377</x:v>
+        <x:v>373</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="49" t="s">
-        <x:v>378</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="B16" s="50" t="s">
-        <x:v>379</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="C16" s="51" t="s">
-        <x:v>380</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="D16" s="50" t="s">
-        <x:v>351</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="E16" s="48" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="F16" s="51" t="s">
-        <x:v>381</x:v>
+        <x:v>377</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="52" t="s">
-        <x:v>382</x:v>
+        <x:v>378</x:v>
       </x:c>
       <x:c r="B17" s="53" t="s">
-        <x:v>352</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="C17" s="54" t="s">
-        <x:v>383</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D17" s="53" t="s">
-        <x:v>351</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="E17" s="48" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="F17" s="54" t="s">
-        <x:v>384</x:v>
+        <x:v>380</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1"/>
@@ -13830,21 +13814,21 @@
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>385</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="14" t="s">
-        <x:v>386</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="B3" s="14" t="s">
-        <x:v>387</x:v>
+        <x:v>383</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="55" t="s">
-        <x:v>388</x:v>
+        <x:v>384</x:v>
       </x:c>
       <x:c r="B4" s="58" t="str">
         <x:v>This workbook is reconciled with the repository, founder decisions, and merged PR #1–#3 baseline through August 16, 2026.</x:v>
@@ -13852,71 +13836,71 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="57" t="s">
-        <x:v>389</x:v>
+        <x:v>385</x:v>
       </x:c>
       <x:c r="B5" s="58" t="s">
-        <x:v>390</x:v>
+        <x:v>386</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="55" t="s">
-        <x:v>391</x:v>
+        <x:v>387</x:v>
       </x:c>
       <x:c r="B6" s="56" t="s">
-        <x:v>392</x:v>
+        <x:v>388</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="57" t="s">
-        <x:v>393</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="B7" s="58" t="s">
-        <x:v>394</x:v>
+        <x:v>390</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="55" t="s">
-        <x:v>395</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="B8" s="56" t="s">
-        <x:v>396</x:v>
+        <x:v>392</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="57" t="s">
-        <x:v>397</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="B9" s="58" t="s">
-        <x:v>398</x:v>
+        <x:v>394</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="55" t="s">
-        <x:v>399</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="B10" s="56" t="s">
-        <x:v>400</x:v>
+        <x:v>396</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="57" t="s">
-        <x:v>401</x:v>
+        <x:v>397</x:v>
       </x:c>
       <x:c r="B11" s="58" t="s">
-        <x:v>402</x:v>
+        <x:v>398</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="55" t="s">
-        <x:v>403</x:v>
+        <x:v>399</x:v>
       </x:c>
       <x:c r="B12" s="56" t="s">
-        <x:v>404</x:v>
+        <x:v>400</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="57" t="s">
-        <x:v>405</x:v>
+        <x:v>401</x:v>
       </x:c>
       <x:c r="B13" s="58" t="str">
         <x:v>Phase 6 expanded — added: NSFW toggle, Settings, Help/Support, Activity, modal/drawer/chat fixes, creator dashboard.</x:v>
@@ -13924,7 +13908,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="55" t="s">
-        <x:v>406</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="B14" s="56" t="str">
         <x:v>Midnight City is implemented as the second free default theme alongside Sakura Kiss, with browser-local selection.</x:v>
@@ -13932,55 +13916,55 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="57" t="s">
-        <x:v>407</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="B15" s="58" t="s">
-        <x:v>408</x:v>
+        <x:v>404</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="5" t="s">
-        <x:v>409</x:v>
+        <x:v>405</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B18" s="60" t="s">
-        <x:v>411</x:v>
+        <x:v>407</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B19" s="60" t="s">
-        <x:v>412</x:v>
+        <x:v>408</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B20" s="60" t="s">
-        <x:v>413</x:v>
+        <x:v>409</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1">
       <x:c r="A21" s="59" t="s">
+        <x:v>406</x:v>
+      </x:c>
+      <x:c r="B21" s="60" t="s">
         <x:v>410</x:v>
-      </x:c>
-      <x:c r="B21" s="60" t="s">
-        <x:v>414</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15.75" customHeight="1">
       <x:c r="A22" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B22" s="60" t="s">
-        <x:v>415</x:v>
+        <x:v>411</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15.75" customHeight="1">
@@ -13989,23 +13973,23 @@
     </x:row>
     <x:row r="24" ht="15.75" customHeight="1">
       <x:c r="A24" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B24" s="60" t="s">
-        <x:v>416</x:v>
+        <x:v>412</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15.75" customHeight="1">
       <x:c r="A25" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B25" s="60" t="s">
-        <x:v>417</x:v>
+        <x:v>413</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15.75" customHeight="1">
       <x:c r="A26" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B26" s="60" t="str">
         <x:v>CCBill is the intended primary processor. Sales has replied; merchant/model approval and technical integration remain pending.</x:v>
@@ -14013,7 +13997,7 @@
     </x:row>
     <x:row r="27" ht="15.75" customHeight="1">
       <x:c r="A27" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B27" s="60" t="str">
         <x:v>Epoch is the intended fallback. Outreach and account-specific cascade confirmation remain pending; no routing is implemented.</x:v>
@@ -14021,31 +14005,31 @@
     </x:row>
     <x:row r="28" ht="15.75" customHeight="1">
       <x:c r="A28" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B28" s="60" t="s">
-        <x:v>418</x:v>
+        <x:v>414</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15.75" customHeight="1">
       <x:c r="A29" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B29" s="60" t="s">
-        <x:v>419</x:v>
+        <x:v>415</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15.75" customHeight="1">
       <x:c r="A30" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B30" s="60" t="s">
-        <x:v>420</x:v>
+        <x:v>416</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A31" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B31" s="60" t="str">
         <x:v>Admin operations: separate apps/admin shell; no public /admin. Public ADMIN sessions are insufficient for operations access. The dormant review router stays unmounted until signed operations identity, exact provisioning, phishing-resistant hardware-backed assurance, private-origin/CSRF, trusted-proxy, restricted DB-role, audit, and recovery gates pass.</x:v>
@@ -14053,7 +14037,7 @@
     </x:row>
     <x:row r="32" ht="15.75" customHeight="1">
       <x:c r="A32" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B32" s="60" t="str">
         <x:v>Midnight City: blue city rooftops, static desktop/mobile JPGs. Browser-local Settings selection implemented; account sync pending.</x:v>
@@ -14061,71 +14045,71 @@
     </x:row>
     <x:row r="33" ht="15.75" customHeight="1">
       <x:c r="A33" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B33" s="60" t="s">
-        <x:v>421</x:v>
+        <x:v>417</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15.75" customHeight="1">
       <x:c r="A34" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B34" s="60" t="s">
-        <x:v>422</x:v>
+        <x:v>418</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15.75" customHeight="1">
       <x:c r="A35" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B35" s="60" t="s">
-        <x:v>423</x:v>
+        <x:v>419</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15.75" customHeight="1">
       <x:c r="A36" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B36" s="60" t="s">
-        <x:v>424</x:v>
+        <x:v>420</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15.75" customHeight="1">
       <x:c r="A37" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B37" s="60" t="s">
-        <x:v>425</x:v>
+        <x:v>421</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15.75" customHeight="1">
       <x:c r="A38" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B38" s="60" t="s">
-        <x:v>426</x:v>
+        <x:v>422</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15.75" customHeight="1">
       <x:c r="A39" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B39" s="60" t="s">
-        <x:v>427</x:v>
+        <x:v>423</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15.75" customHeight="1">
       <x:c r="A40" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B40" s="60" t="s">
-        <x:v>428</x:v>
+        <x:v>424</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15.75" customHeight="1">
       <x:c r="A41" s="59" t="s">
-        <x:v>410</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="B41" s="60" t="inlineStr">
         <x:is>
@@ -15664,7 +15648,7 @@
   <x:sheetData>
     <x:row r="1" ht="39.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>429</x:v>
+        <x:v>425</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -15688,22 +15672,22 @@
     </x:row>
     <x:row r="3" ht="25.5" customHeight="1">
       <x:c r="A3" s="68" t="s">
+        <x:v>426</x:v>
+      </x:c>
+      <x:c r="B3" s="68" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="C3" s="68" t="s">
+        <x:v>427</x:v>
+      </x:c>
+      <x:c r="D3" s="68" t="s">
+        <x:v>428</x:v>
+      </x:c>
+      <x:c r="E3" s="68" t="s">
+        <x:v>429</x:v>
+      </x:c>
+      <x:c r="F3" s="68" t="s">
         <x:v>430</x:v>
-      </x:c>
-      <x:c r="B3" s="68" t="s">
-        <x:v>332</x:v>
-      </x:c>
-      <x:c r="C3" s="68" t="s">
-        <x:v>431</x:v>
-      </x:c>
-      <x:c r="D3" s="68" t="s">
-        <x:v>432</x:v>
-      </x:c>
-      <x:c r="E3" s="68" t="s">
-        <x:v>433</x:v>
-      </x:c>
-      <x:c r="F3" s="68" t="s">
-        <x:v>434</x:v>
       </x:c>
       <x:c r="G3" s="68" t="s">
         <x:v>4</x:v>
@@ -15714,7 +15698,7 @@
     </x:row>
     <x:row r="4" ht="25.5" customHeight="1">
       <x:c r="A4" s="15" t="s">
-        <x:v>435</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -15726,98 +15710,98 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="16" t="s">
-        <x:v>436</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="B5" s="17" t="s">
-        <x:v>437</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="C5" s="17" t="s">
-        <x:v>438</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="D5" s="17">
         <x:v>500.0</x:v>
       </x:c>
       <x:c r="E5" s="17"/>
       <x:c r="F5" s="17" t="s">
-        <x:v>439</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="G5" s="24" t="s">
-        <x:v>440</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="H5" s="17" t="s">
-        <x:v>441</x:v>
+        <x:v>437</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="20" t="s">
-        <x:v>442</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="B6" s="21" t="s">
-        <x:v>437</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="C6" s="21" t="s">
-        <x:v>438</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="D6" s="21">
         <x:v>500.0</x:v>
       </x:c>
       <x:c r="E6" s="21"/>
       <x:c r="F6" s="21" t="s">
+        <x:v>435</x:v>
+      </x:c>
+      <x:c r="G6" s="24" t="s">
+        <x:v>436</x:v>
+      </x:c>
+      <x:c r="H6" s="21" t="s">
         <x:v>439</x:v>
-      </x:c>
-      <x:c r="G6" s="24" t="s">
-        <x:v>440</x:v>
-      </x:c>
-      <x:c r="H6" s="21" t="s">
-        <x:v>443</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="16" t="s">
-        <x:v>444</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="B7" s="17" t="s">
-        <x:v>437</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="C7" s="17" t="s">
-        <x:v>438</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="D7" s="17">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E7" s="17"/>
       <x:c r="F7" s="17" t="s">
-        <x:v>439</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="G7" s="24" t="s">
-        <x:v>440</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="H7" s="17" t="s">
-        <x:v>445</x:v>
+        <x:v>441</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="20" t="s">
-        <x:v>446</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="B8" s="21" t="s">
-        <x:v>447</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="C8" s="21" t="s">
-        <x:v>438</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="D8" s="21">
         <x:v>350.0</x:v>
       </x:c>
       <x:c r="E8" s="21"/>
       <x:c r="F8" s="21" t="s">
-        <x:v>439</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="G8" s="24" t="s">
-        <x:v>440</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="H8" s="21" t="s">
-        <x:v>448</x:v>
+        <x:v>444</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -15835,10 +15819,10 @@
         <x:v>Kiban Digital Holdings LLC — Northwest formation</x:v>
       </x:c>
       <x:c r="B10" s="208" t="s">
-        <x:v>447</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="C10" s="208" t="s">
-        <x:v>438</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="D10" s="208">
         <x:v>155.0</x:v>
@@ -15847,7 +15831,7 @@
         <x:v>196</x:v>
       </x:c>
       <x:c r="F10" s="208" t="s">
-        <x:v>439</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="G10" s="213" t="str">
         <x:v>Paid / filed</x:v>
@@ -15861,10 +15845,10 @@
         <x:v>Policy documents — Suzanne Lawyer (Fiverr)</x:v>
       </x:c>
       <x:c r="B11" s="208" t="s">
-        <x:v>447</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="C11" s="208" t="s">
-        <x:v>438</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="D11" s="208">
         <x:v>125.0</x:v>
@@ -15873,7 +15857,7 @@
         <x:v>1100</x:v>
       </x:c>
       <x:c r="F11" s="208" t="s">
-        <x:v>439</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="G11" s="214" t="str">
         <x:v>Paid / drafting</x:v>
@@ -15884,79 +15868,79 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="16" t="s">
-        <x:v>449</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="B12" s="17" t="s">
-        <x:v>447</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="C12" s="17" t="s">
-        <x:v>450</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="D12" s="17">
         <x:v>125.0</x:v>
       </x:c>
       <x:c r="E12" s="17"/>
       <x:c r="F12" s="17" t="s">
-        <x:v>451</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="G12" s="24" t="s">
-        <x:v>440</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="H12" s="17" t="s">
-        <x:v>452</x:v>
+        <x:v>448</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="20" t="s">
-        <x:v>453</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="B13" s="21" t="s">
-        <x:v>454</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="C13" s="21" t="s">
-        <x:v>450</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="D13" s="21">
         <x:v>15.0</x:v>
       </x:c>
       <x:c r="E13" s="21"/>
       <x:c r="F13" s="21" t="s">
+        <x:v>447</x:v>
+      </x:c>
+      <x:c r="G13" s="24" t="s">
+        <x:v>436</x:v>
+      </x:c>
+      <x:c r="H13" s="21" t="s">
         <x:v>451</x:v>
-      </x:c>
-      <x:c r="G13" s="24" t="s">
-        <x:v>440</x:v>
-      </x:c>
-      <x:c r="H13" s="21" t="s">
-        <x:v>455</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="16.5" customHeight="1">
       <x:c r="A14" s="16" t="s">
-        <x:v>456</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="B14" s="17" t="s">
-        <x:v>454</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="C14" s="17" t="s">
-        <x:v>450</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="D14" s="17">
         <x:v>30.0</x:v>
       </x:c>
       <x:c r="E14" s="17"/>
       <x:c r="F14" s="17" t="s">
-        <x:v>451</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="G14" s="24" t="s">
-        <x:v>440</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="H14" s="17" t="s">
-        <x:v>457</x:v>
+        <x:v>453</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="15" t="s">
-        <x:v>458</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="B15" s="2"/>
       <x:c r="C15" s="2"/>
@@ -15968,175 +15952,175 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="32" t="s">
-        <x:v>459</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="B16" s="33" t="s">
-        <x:v>454</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="C16" s="33" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="D16" s="33">
         <x:v>18.0</x:v>
       </x:c>
       <x:c r="E16" s="33"/>
       <x:c r="F16" s="33" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="G16" s="39" t="s">
-        <x:v>440</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="H16" s="33" t="s">
-        <x:v>461</x:v>
+        <x:v>457</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="20" t="s">
-        <x:v>462</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="B17" s="21" t="s">
-        <x:v>454</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="C17" s="21" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="D17" s="21">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E17" s="21"/>
       <x:c r="F17" s="21" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="G17" s="24" t="s">
-        <x:v>440</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="H17" s="21" t="s">
-        <x:v>463</x:v>
+        <x:v>459</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="16" t="s">
-        <x:v>464</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="B18" s="17" t="s">
-        <x:v>454</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="C18" s="17" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="D18" s="17">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E18" s="17"/>
       <x:c r="F18" s="17" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="G18" s="24" t="s">
-        <x:v>440</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="H18" s="17" t="s">
-        <x:v>465</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="20" t="s">
-        <x:v>466</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="B19" s="21" t="s">
-        <x:v>454</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="C19" s="21" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="D19" s="21">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E19" s="21"/>
       <x:c r="F19" s="21" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="G19" s="24" t="s">
-        <x:v>440</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="H19" s="21" t="s">
-        <x:v>467</x:v>
+        <x:v>463</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="16" t="s">
-        <x:v>468</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="B20" s="17" t="s">
-        <x:v>454</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="C20" s="17" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="D20" s="17">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E20" s="17"/>
       <x:c r="F20" s="17" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="G20" s="24" t="s">
-        <x:v>440</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="H20" s="17" t="s">
-        <x:v>469</x:v>
+        <x:v>465</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1">
       <x:c r="A21" s="20" t="s">
-        <x:v>470</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="B21" s="21" t="s">
-        <x:v>454</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="C21" s="21" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="D21" s="21">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E21" s="21"/>
       <x:c r="F21" s="21" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="G21" s="24" t="s">
-        <x:v>440</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="H21" s="21" t="s">
-        <x:v>471</x:v>
+        <x:v>467</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="25.5" customHeight="1">
       <x:c r="A22" s="36" t="s">
-        <x:v>472</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="B22" s="37" t="s">
-        <x:v>454</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="C22" s="37" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="D22" s="37">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E22" s="37"/>
       <x:c r="F22" s="37" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="G22" s="30" t="s">
-        <x:v>440</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="H22" s="37" t="s">
-        <x:v>473</x:v>
+        <x:v>469</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15.75" customHeight="1">
       <x:c r="A23" s="15" t="s">
-        <x:v>474</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="B23" s="2"/>
       <x:c r="C23" s="2"/>
@@ -16148,79 +16132,79 @@
     </x:row>
     <x:row r="24" ht="15.75" customHeight="1">
       <x:c r="A24" s="32" t="s">
-        <x:v>475</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="B24" s="33" t="s">
-        <x:v>437</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="C24" s="33" t="s">
-        <x:v>476</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="D24" s="33">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E24" s="33"/>
       <x:c r="F24" s="33" t="s">
-        <x:v>477</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="G24" s="39" t="s">
-        <x:v>478</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="H24" s="33" t="s">
-        <x:v>479</x:v>
+        <x:v>475</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15.75" customHeight="1">
       <x:c r="A25" s="20" t="s">
-        <x:v>480</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="B25" s="21" t="s">
-        <x:v>437</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="C25" s="21" t="s">
-        <x:v>476</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="D25" s="21">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E25" s="21"/>
       <x:c r="F25" s="21" t="s">
+        <x:v>473</x:v>
+      </x:c>
+      <x:c r="G25" s="24" t="s">
+        <x:v>474</x:v>
+      </x:c>
+      <x:c r="H25" s="21" t="s">
         <x:v>477</x:v>
-      </x:c>
-      <x:c r="G25" s="24" t="s">
-        <x:v>478</x:v>
-      </x:c>
-      <x:c r="H25" s="21" t="s">
-        <x:v>481</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="25.5" customHeight="1">
       <x:c r="A26" s="36" t="s">
-        <x:v>482</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="B26" s="37" t="s">
-        <x:v>437</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="C26" s="37" t="s">
-        <x:v>476</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="D26" s="37">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E26" s="37"/>
       <x:c r="F26" s="37" t="s">
-        <x:v>483</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="G26" s="30" t="s">
-        <x:v>478</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="H26" s="37" t="s">
-        <x:v>484</x:v>
+        <x:v>480</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15.75" customHeight="1">
       <x:c r="A27" s="15" t="s">
-        <x:v>485</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="B27" s="2"/>
       <x:c r="C27" s="2"/>
@@ -16232,80 +16216,80 @@
     </x:row>
     <x:row r="28" ht="15.75" customHeight="1">
       <x:c r="A28" s="32" t="s">
-        <x:v>486</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="B28" s="33" t="s">
-        <x:v>437</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="C28" s="33" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="D28" s="33">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E28" s="33"/>
       <x:c r="F28" s="33" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="G28" s="39" t="s">
-        <x:v>487</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="H28" s="33" t="s">
-        <x:v>488</x:v>
+        <x:v>484</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15.75" customHeight="1">
       <x:c r="A29" s="20" t="s">
-        <x:v>489</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="B29" s="21" t="s">
-        <x:v>490</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="C29" s="21" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="D29" s="21">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E29" s="21"/>
       <x:c r="F29" s="21" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="G29" s="24" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="H29" s="21" t="s">
         <x:v>487</x:v>
-      </x:c>
-      <x:c r="H29" s="21" t="s">
-        <x:v>491</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15.75" customHeight="1">
       <x:c r="A30" s="16" t="s">
-        <x:v>492</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="B30" s="17" t="s">
-        <x:v>447</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="C30" s="17" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="D30" s="17">
         <x:v>0.0</x:v>
       </x:c>
       <x:c r="E30" s="17"/>
       <x:c r="F30" s="17" t="s">
-        <x:v>460</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="G30" s="24" t="s">
-        <x:v>487</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="H30" s="17" t="s">
-        <x:v>493</x:v>
+        <x:v>489</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="25.5" customHeight="1"/>
     <x:row r="32" ht="15.75" customHeight="1">
       <x:c r="A32" s="15" t="s">
-        <x:v>494</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="B32" s="2"/>
       <x:c r="C32" s="2"/>
@@ -16317,7 +16301,7 @@
     </x:row>
     <x:row r="33" ht="15.75" customHeight="1">
       <x:c r="A33" s="6" t="s">
-        <x:v>495</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="B33" s="69" t="n">
         <x:f>SUM(D5:D11)</x:f>
@@ -16326,7 +16310,7 @@
     </x:row>
     <x:row r="34" ht="15.75" customHeight="1">
       <x:c r="A34" s="7" t="s">
-        <x:v>496</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="B34" s="70" t="n">
         <x:f>SUM(D12:D14)</x:f>
@@ -16335,7 +16319,7 @@
     </x:row>
     <x:row r="35" ht="15.75" customHeight="1">
       <x:c r="A35" s="6" t="s">
-        <x:v>497</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="B35" s="69" t="n">
         <x:f>SUM(D16:D22)</x:f>
@@ -16344,7 +16328,7 @@
     </x:row>
     <x:row r="36" ht="15.75" customHeight="1">
       <x:c r="A36" s="7" t="s">
-        <x:v>498</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="B36" s="70" t="n">
         <x:f>B33+B34+B35*12</x:f>
@@ -17375,7 +17359,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="s">
-        <x:v>499</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="B1"/>
       <x:c r="C1"/>
@@ -17386,7 +17370,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="s">
-        <x:v>500</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="B2"/>
       <x:c r="C2"/>
@@ -17406,12 +17390,12 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="s">
-        <x:v>501</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="B4"/>
       <x:c r="C4"/>
       <x:c r="D4" t="s">
-        <x:v>502</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="E4"/>
       <x:c r="F4"/>
@@ -17419,7 +17403,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="s">
-        <x:v>503</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="B5" t="n">
         <x:f>COUNTIF('Master Tracker'!C4:C164,"✅ Done")+COUNTIF('Master Tracker'!C4:C164,"🔄 In Progress")+COUNTIF('Master Tracker'!C4:C164,"📋 Not Started")</x:f>
@@ -17427,11 +17411,11 @@
       </x:c>
       <x:c r="C5"/>
       <x:c r="D5" t="s">
-        <x:v>504</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="E5" t="n">
         <x:f>COUNTA(Backlog!A2:A30)</x:f>
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F5"/>
       <x:c r="G5"/>
@@ -17450,7 +17434,7 @@
       </x:c>
       <x:c r="E6" t="n">
         <x:f>COUNTIF(Backlog!E2:E30,"📋 Not Started")</x:f>
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F6"/>
       <x:c r="G6"/>
@@ -17461,7 +17445,7 @@
       </x:c>
       <x:c r="B7" t="n">
         <x:f>COUNTIF('Master Tracker'!C4:C164,"🔄 In Progress")</x:f>
-        <x:v>51</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C7"/>
       <x:c r="D7"/>
@@ -17475,7 +17459,7 @@
       </x:c>
       <x:c r="B8" t="n">
         <x:f>COUNTIF('Master Tracker'!C4:C164,"📋 Not Started")</x:f>
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C8"/>
       <x:c r="D8"/>
@@ -17485,7 +17469,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="s">
-        <x:v>505</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="B9" t="n">
         <x:f>IF(B5=0,0,B6/B5)</x:f>
@@ -17517,11 +17501,11 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="s">
-        <x:v>506</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="B12"/>
       <x:c r="C12" t="s">
-        <x:v>507</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="D12"/>
       <x:c r="E12"/>
@@ -17547,7 +17531,7 @@
       </x:c>
       <x:c r="B14"/>
       <x:c r="C14" t="s">
-        <x:v>508</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="D14"/>
       <x:c r="E14"/>
@@ -17560,7 +17544,7 @@
       </x:c>
       <x:c r="B15"/>
       <x:c r="C15" t="s">
-        <x:v>509</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="D15"/>
       <x:c r="E15"/>
@@ -17571,7 +17555,7 @@
       <x:c r="A16"/>
       <x:c r="B16"/>
       <x:c r="C16" t="s">
-        <x:v>510</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="D16"/>
       <x:c r="E16"/>
@@ -17582,7 +17566,7 @@
       <x:c r="A17"/>
       <x:c r="B17"/>
       <x:c r="C17" t="s">
-        <x:v>511</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="D17"/>
       <x:c r="E17"/>
@@ -17593,7 +17577,7 @@
       <x:c r="A18"/>
       <x:c r="B18"/>
       <x:c r="C18" t="s">
-        <x:v>512</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="D18"/>
       <x:c r="E18"/>
@@ -17604,7 +17588,7 @@
       <x:c r="A19"/>
       <x:c r="B19"/>
       <x:c r="C19" t="s">
-        <x:v>513</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="D19"/>
       <x:c r="E19"/>
@@ -18841,15 +18825,15 @@
       </x:c>
       <x:c r="F12" s="111" t="n">
         <x:f>COUNTIF('Delivery Tracker'!$B$4:$B$400,$A12)</x:f>
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G12" s="119" t="n">
         <x:f>IF(F12=0,0,E12/F12)</x:f>
-        <x:v>0.4444444444444444</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="H12" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A12,'Delivery Tracker'!$H$4:$H$400,"In Progress")</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="I12" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A12,'Delivery Tracker'!$H$4:$H$400,"In Review")</x:f>
@@ -18864,19 +18848,19 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L12" s="111" t="str">
-        <x:v>Connect discovery, Store and feed remain launch scope. Connect means online, price and language filters.</x:v>
+        <x:v>Feed, Store and Connect remain launch scope (online/price/language discovery). Your Activity /activity UI is an explicit example-data preview; real member history remains pending.</x:v>
       </x:c>
       <x:c r="M12" s="111" t="str">
-        <x:v>Integrate content and access controls. Define service/order and beta payment rules with the relevant slice.</x:v>
+        <x:v>Integrate content/access, service/order and beta payment rules. Connect Your Activity to authenticated P05/P06/P07 data.</x:v>
       </x:c>
       <x:c r="N12" s="111" t="str">
-        <x:v>Feed actions persist; Store uses real data; creator discovery filters work. Separately define service order/payment rules.</x:v>
+        <x:v>Feed actions persist; Store and Your Activity use real account data; creator discovery filters work. Service/order/payment rules separately defined.</x:v>
       </x:c>
       <x:c r="O12" s="111" t="str">
         <x:v>https://github.com/QK-Connoisseur/PDoki/blob/dev/PLAN.md#12-phase-8--feed-social-actions-store-and-connect</x:v>
       </x:c>
       <x:c r="P12" s="112" t="n">
-        <x:v>46274.666666666664</x:v>
+        <x:v>46275.666666666664</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
@@ -19240,7 +19224,7 @@
       </x:c>
       <x:c r="F19" s="111" t="n">
         <x:f>COUNTIF('Delivery Tracker'!$B$4:$B$400,$A19)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G19" s="119" t="n">
         <x:f>IF(F19=0,0,E19/F19)</x:f>
@@ -19260,7 +19244,7 @@
       </x:c>
       <x:c r="K19" s="111" t="n">
         <x:f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A19,'Delivery Tracker'!$H$4:$H$400,"Not Started")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L19" s="111" t="str">
         <x:v>Live streaming, advanced recommendations, native apps, crypto, extra themes, and advanced group chat remain deferred.</x:v>
@@ -19301,7 +19285,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68c94d1baaac45d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1018c19920934ead"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23037,50 +23021,54 @@
         <x:v>LEG-MT-080</x:v>
       </x:c>
       <x:c r="B74" s="111" t="str">
-        <x:v>POST</x:v>
+        <x:v>P08</x:v>
       </x:c>
       <x:c r="C74" s="111" t="str">
-        <x:v>Post-MVP</x:v>
-      </x:c>
-      <x:c r="D74" s="111" t="str"/>
+        <x:v>Feed, social actions, Store, and Connect</x:v>
+      </x:c>
+      <x:c r="D74" s="111" t="str">
+        <x:v>P03, P05, P06, P07</x:v>
+      </x:c>
       <x:c r="E74" s="111" t="str">
         <x:v>Legacy-mapped task</x:v>
       </x:c>
       <x:c r="F74" s="111" t="str">
-        <x:v>Post-MVP</x:v>
+        <x:v>Feed, social actions, Store, and Connect</x:v>
       </x:c>
       <x:c r="G74" s="111" t="str">
         <x:v>Build 'Your Activity' page</x:v>
       </x:c>
       <x:c r="H74" s="111" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="I74" s="111" t="str">
-        <x:v>N/A</x:v>
+        <x:v>UI Prototype</x:v>
       </x:c>
       <x:c r="J74" s="111" t="str">
-        <x:v>Low</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="K74" s="111" t="str">
         <x:v>Engineering</x:v>
       </x:c>
       <x:c r="L74" s="111" t="str"/>
       <x:c r="M74" s="111" t="str">
-        <x:v>Confirm dependencies and owner, then define the first deliverable.</x:v>
+        <x:v>Connect authenticated API and persisted member history after P05/P06/P07. Replace example data when real event sources exist.</x:v>
       </x:c>
       <x:c r="N74" s="112"/>
-      <x:c r="O74" s="111" t="str"/>
+      <x:c r="O74" s="111" t="str">
+        <x:v>apps/web/src/pages/ActivityPage.jsx; ActivityPage.test.jsx; tests/e2e/activity.spec.js; PLAN.md §12.</x:v>
+      </x:c>
       <x:c r="P74" s="112" t="n">
-        <x:v>46250.666666666664</x:v>
+        <x:v>46275.666666666664</x:v>
       </x:c>
       <x:c r="Q74" s="111" t="str">
-        <x:v>Member activity history: posts liked, content purchased, subscriptions and payment history. Lower priority.</x:v>
+        <x:v>P08 member history: liked posts, purchases, subscriptions and payment history. UI preview first; account-backed events follow.</x:v>
       </x:c>
       <x:c r="R74" s="111" t="str">
-        <x:v>Nice-to-have post-launch. Defer if time is tight.</x:v>
+        <x:v>Promoted from Post-MVP to P08. /activity preview provides search/category filters and sidebar/header Your Activity links. Example data is explicitly labeled; authenticated account data, API and persistence remain pending. Focused UI tests passed.</x:v>
       </x:c>
       <x:c r="S74" s="111" t="str">
-        <x:v>Preserved Master Tracker row 80; legacy status: 📋 Not Started</x:v>
+        <x:v>Master Tracker row 80; promoted to P08 September 10, 2026. Former duplicate Backlog row 14 cleared.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="46" customHeight="1">
@@ -27734,7 +27722,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38016ecd093840d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48f51c6e063b438b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record questionnaire decisions and Founders benefits
</commit_message>
<xml_diff>
--- a/docs/product/Pumdoki_MasterTracker_V4.xlsx
+++ b/docs/product/Pumdoki_MasterTracker_V4.xlsx
@@ -7014,8 +7014,8 @@
       <c r="N1" s="94"/>
     </row>
     <row r="2" spans="1:14" ht="21.75" customHeight="1">
-      <c r="A2" s="95" t="s">
-        <v>511</v>
+      <c r="A2" t="str" s="95">
+        <v>Updated September 16, 2026. Founder confirms Maryland approval and EIN receipt. Private R2 flow verified; local content review remains pending. Record counts are not launch readiness.</v>
       </c>
       <c r="B2" s="95"/>
       <c r="C2" s="95"/>
@@ -7183,12 +7183,12 @@
       <c r="B13" s="102"/>
       <c r="C13" s="101">
         <f>COUNTIF('Delivery Tracker'!$H$4:$H$400,"Done")</f>
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D13" s="102"/>
       <c r="E13" s="101">
         <f>COUNTIF('Delivery Tracker'!$H$4:$H$400,"In Progress")</f>
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F13" s="102"/>
       <c r="G13" s="101">
@@ -7208,7 +7208,7 @@
       <c r="L13" s="102"/>
       <c r="M13" s="105">
         <f>IF(A13=0,0,C13/A13)</f>
-        <v>0.20512820512820512</v>
+        <v>0.21153846153846154</v>
       </c>
       <c r="N13" s="102"/>
     </row>
@@ -7542,7 +7542,7 @@
       </c>
       <c r="E22" s="62">
         <f>'Phase Roadmap'!E8</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F22" s="62">
         <f>'Phase Roadmap'!F8</f>
@@ -7550,11 +7550,11 @@
       </c>
       <c r="G22" s="65">
         <f>'Phase Roadmap'!G8</f>
-        <v>0.14285714285714285</v>
+        <v>0.17142857142857143</v>
       </c>
       <c r="H22" s="62">
         <f>'Phase Roadmap'!H8</f>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I22" s="62">
         <f>'Phase Roadmap'!I8</f>
@@ -7570,7 +7570,7 @@
       </c>
       <c r="L22" s="62" t="str">
         <f>'Phase Roadmap'!L8</f>
-        <v>Slices 1–4 published; operations dormant. Maryland approval pending. Initial CCBill reply retained; proposed follow-up cancelled. Founder/provider work now accompanies each functional code slice.</v>
+        <v>Slices 1-4 published; operations dormant. Founder confirms Maryland approval and EIN receipt Sept 16. Legal review and business/provider dependencies remain open.</v>
       </c>
       <c r="M22" s="62" t="str">
         <f>'Phase Roadmap'!M8</f>
@@ -10023,19 +10023,43 @@
         </is>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="57.95" customHeight="1">
-      <c r="A12" s="62"/>
-      <c r="B12" s="62"/>
-      <c r="C12" s="62"/>
-      <c r="D12" s="62"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="62"/>
-      <c r="G12" s="62"/>
-      <c r="H12" s="62"/>
-      <c r="I12" s="62"/>
-      <c r="J12" s="62"/>
-      <c r="K12" s="62"/>
-      <c r="L12" s="62"/>
+    <row r="12" spans="1:12" ht="85" customHeight="1">
+      <c r="A12" t="n" s="63">
+        <v>46281</v>
+      </c>
+      <c r="B12" t="str" s="62">
+        <v>LEG-MT-158</v>
+      </c>
+      <c r="C12" t="str" s="62">
+        <v>P04</v>
+      </c>
+      <c r="D12" t="str" s="62">
+        <v>Record Maryland approval and EIN receipt.</v>
+      </c>
+      <c r="E12" t="str" s="62">
+        <v>Marked LLC formation complete; updated EIN, privacy and dependency records.</v>
+      </c>
+      <c r="F12" t="str" s="62">
+        <v>State formation and EIN are complete, per founder confirmation.</v>
+      </c>
+      <c r="G12" t="str" s="62">
+        <v>Banking, DBA and processor approval remain open. Product readiness unchanged.</v>
+      </c>
+      <c r="H12" t="str" s="62">
+        <v>Founder confirmed approval and supplied EIN in chat September 16, 2026.</v>
+      </c>
+      <c r="I12" t="str" s="62">
+        <v>Done</v>
+      </c>
+      <c r="J12" t="str" s="62">
+        <v>Original approval and IRS letter not independently inspected.</v>
+      </c>
+      <c r="K12" t="str" s="62">
+        <v>Resume the current legal questionnaire in PLAN.md section 20.</v>
+      </c>
+      <c r="L12" t="str" s="62">
+        <v>Codex</v>
+      </c>
     </row>
     <row r="13" spans="1:12" ht="57.95" customHeight="1">
       <c r="A13" s="62"/>
@@ -11016,27 +11040,27 @@
       <c r="B9" s="62" t="s">
         <v>829</v>
       </c>
-      <c r="C9" s="62" t="s">
-        <v>1577</v>
+      <c r="C9" t="str" s="62">
+        <v>Maryland LLC approved; EIN obtained</v>
       </c>
       <c r="D9" s="62" t="s">
         <v>808</v>
       </c>
       <c r="E9" s="63"/>
-      <c r="F9" s="62" t="s">
-        <v>529</v>
-      </c>
-      <c r="G9" s="62" t="s">
-        <v>1578</v>
-      </c>
-      <c r="H9" s="62" t="s">
-        <v>1579</v>
-      </c>
-      <c r="I9" s="62" t="s">
-        <v>1580</v>
-      </c>
-      <c r="J9" s="63">
-        <v>46275.666666666664</v>
+      <c r="F9" t="str" s="62">
+        <v>Done</v>
+      </c>
+      <c r="G9" t="str" s="62">
+        <v>Founder confirmed Maryland approval and EIN receipt Sept 16. Northwest formation cost: $196. Banking and DBA remain open.</v>
+      </c>
+      <c r="H9" t="str" s="62">
+        <v>Retain state approval and IRS confirmation privately. Resume the existing legal questionnaire; handle banking and DBA separately.</v>
+      </c>
+      <c r="I9" t="str" s="62">
+        <v>Founder confirmation, September 16, 2026. EIN supplied in chat; originals not independently inspected. $196 cost previously confirmed September 10.</v>
+      </c>
+      <c r="J9" t="n" s="63">
+        <v>46281</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="54.95" customHeight="1">
@@ -11088,15 +11112,17 @@
       <c r="F11" s="62" t="s">
         <v>531</v>
       </c>
-      <c r="G11" s="62" t="s">
-        <v>1587</v>
-      </c>
-      <c r="H11" s="62" t="s">
-        <v>1588</v>
-      </c>
-      <c r="I11" s="62"/>
-      <c r="J11" s="63">
-        <v>46255.666666666664</v>
+      <c r="G11" s="62" t="str">
+        <v>Automated member age assurance and creator identity checks planned. Ondato/Veriff candidates; selection, total costs, country coverage and privacy/retention terms remain unresolved.</v>
+      </c>
+      <c r="H11" s="62" t="str">
+        <v>Compare candidates against pilot needs and CCBill review requirements. Configure/test required flows before live adult access or real creator identity onboarding.</v>
+      </c>
+      <c r="I11" s="62" t="str">
+        <v>Founder approval Sept 13; PLAN.md §3.5/§20, Question 12.</v>
+      </c>
+      <c r="J11" s="63" t="n">
+        <v>46278</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="54.95" customHeight="1">
@@ -11148,17 +11174,17 @@
       <c r="F13" s="62" t="s">
         <v>531</v>
       </c>
-      <c r="G13" s="62" t="s">
-        <v>1595</v>
-      </c>
-      <c r="H13" s="62" t="s">
-        <v>1596</v>
-      </c>
-      <c r="I13" s="62" t="s">
-        <v>1597</v>
-      </c>
-      <c r="J13" s="63">
-        <v>46255.666666666664</v>
+      <c r="G13" s="62" t="str">
+        <v>Maryland operator; broad international creators and limited international member pilot approved. Automated checks/cash buffer planned; countries, limits, budgets and coverage unresolved.</v>
+      </c>
+      <c r="H13" s="62" t="str">
+        <v>Set pilot member cap, verification budget and cash buffer before live use; verify actual country coverage. Resolve creator tax documentation under LEG-MT-021.</v>
+      </c>
+      <c r="I13" s="62" t="str">
+        <v>PLAN.md §3.6/§20, Q9–10 (Sept 13 approval); docs/product/initial-business-definition.md (Sept 6 review).</v>
+      </c>
+      <c r="J13" s="63" t="n">
+        <v>46278</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="54.95" customHeight="1">
@@ -11180,17 +11206,17 @@
       <c r="F14" s="62" t="s">
         <v>531</v>
       </c>
-      <c r="G14" s="62" t="s">
-        <v>1600</v>
-      </c>
-      <c r="H14" s="62" t="s">
-        <v>1601</v>
-      </c>
-      <c r="I14" s="62" t="s">
-        <v>1597</v>
-      </c>
-      <c r="J14" s="63">
-        <v>46274.666666666664</v>
+      <c r="G14" s="62" t="str">
+        <v>Q131 approves a 20/80 target excluding sales tax; processing costs from platform share. Q132 applies standard fees to Founders, replacing cost-recovery terms.</v>
+      </c>
+      <c r="H14" s="62" t="str">
+        <v>Validate actual costs before firm pricing/live payments. Refund/chargeback allocation and payout fees pending. Budget prize events separately.</v>
+      </c>
+      <c r="I14" s="62" t="str">
+        <v>PLAN.md §3.8 and §20, Q131–132 approved September 22, 2026.</v>
+      </c>
+      <c r="J14" s="63" t="n">
+        <v>46287</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="54.95" customHeight="1">
@@ -11444,8 +11470,8 @@
       <c r="B23" s="69" t="s">
         <v>838</v>
       </c>
-      <c r="C23" s="69" t="s">
-        <v>1637</v>
+      <c r="C23" s="69" t="str">
+        <v>Founders acquisition and benefits</v>
       </c>
       <c r="D23" s="69" t="s">
         <v>808</v>
@@ -11454,17 +11480,17 @@
       <c r="F23" s="69" t="s">
         <v>529</v>
       </c>
-      <c r="G23" s="69" t="s">
-        <v>1638</v>
-      </c>
-      <c r="H23" s="69" t="s">
-        <v>1639</v>
-      </c>
-      <c r="I23" s="69" t="s">
-        <v>1597</v>
-      </c>
-      <c r="J23" s="70">
-        <v>46271.666666666664</v>
+      <c r="G23" s="69" t="str">
+        <v>Q132: Founders tag; Connect filter or Explore section below top sections; SFW Discord events; future event priority. Standard fees replace commission exemption.</v>
+      </c>
+      <c r="H23" s="69" t="str">
+        <v>Q133: define eligibility, cutoff/cap and duration. Specify placements and event terms; cash prizes optional, separately funded. No sales/ranking guarantee.</v>
+      </c>
+      <c r="I23" s="69" t="str">
+        <v>PLAN.md §20, Q132 approved September 22, 2026; Q133 pending.</v>
+      </c>
+      <c r="J23" s="70" t="n">
+        <v>46287</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="95.1" customHeight="1">
@@ -11916,8 +11942,8 @@
       <c r="C22" s="76">
         <v>300</v>
       </c>
-      <c r="D22" s="71" t="s">
-        <v>1696</v>
+      <c r="D22" t="str" s="71">
+        <v>Specific tax/accounting advice only when needed. Maryland approval and EIN receipt confirmed Sept 16. Unquoted allowance unchanged.</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="48" customHeight="1">
@@ -11946,8 +11972,8 @@
       <c r="C24" s="76">
         <v>900</v>
       </c>
-      <c r="D24" s="71" t="s">
-        <v>1700</v>
+      <c r="D24" t="str" s="71">
+        <v>Northwest formation: $196 confirmed paid. State approval and EIN receipt confirmed Sept 16. Actual recorded in Expense Tracker; planning allowance unchanged.</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="48" customHeight="1">
@@ -12667,8 +12693,8 @@
       <c r="C11" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="8" t="s">
-        <v>27</v>
+      <c r="D11" s="8" t="str">
+        <v>Q34: 60 days; Q35: Maryland venue with mandatory-rights exceptions. Q33 advice, legal copy and live workflows pending. PLAN.md §20.</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -12681,8 +12707,8 @@
       <c r="C12" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="11" t="s">
-        <v>30</v>
+      <c r="D12" s="11" t="str">
+        <v>Q50: international privacy provisions where applicable. Q51 vendor terms pending. Controls/final review pending. PLAN.md §20.</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -12695,8 +12721,8 @@
       <c r="C13" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="8" t="s">
-        <v>33</v>
+      <c r="D13" s="8" t="str">
+        <v>Q75 approved: serious-violation removal aligned with Q62-64. Final policy/controls pending. Active review: LEG-MT-015. PLAN.md §20.</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -12709,8 +12735,8 @@
       <c r="C14" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="11" t="s">
-        <v>36</v>
+      <c r="D14" s="11" t="str">
+        <v>Q64 reporting/preservation approved. AUP review pending; controls unimplemented. Community review: LEG-MT-013. PLAN.md §20.</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="30">
@@ -12723,8 +12749,8 @@
       <c r="C15" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="8" t="s">
-        <v>39</v>
+      <c r="D15" s="8" t="str">
+        <v>Q85 approved: creator notices/warnings, no guaranteed warning count. DMCA draft review done; final policy/controls pending. Active: LEG-MT-028. PLAN.md §20.</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30">
@@ -12737,8 +12763,8 @@
       <c r="C16" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="11" t="s">
-        <v>42</v>
+      <c r="D16" s="11" t="str">
+        <v>Q55: statutory records segregated from consent releases where §2257 applies. Custodian, forms and workflow pending. PLAN.md §20.</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="30">
@@ -12793,8 +12819,8 @@
       <c r="C20" s="91" t="s">
         <v>26</v>
       </c>
-      <c r="D20" s="11" t="s">
-        <v>581</v>
+      <c r="D20" s="11" t="str">
+        <v>Q17 approved: CCBill intake received; no detailed checklist/approval. Use current Mastercard rules; align later. PLAN.md §20.</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="15.75" customHeight="1">
@@ -12804,11 +12830,11 @@
       <c r="B21" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C21" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>56</v>
+      <c r="C21" s="91" t="str">
+        <v>🔄 In Progress</v>
+      </c>
+      <c r="D21" s="8" t="str">
+        <v>Q132 approved: Founders benefits replace fee exemption. Review Q133 duration and eligibility. PLAN.md §20.</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="15.75" customHeight="1">
@@ -12891,8 +12917,8 @@
       <c r="C27" s="91" t="s">
         <v>26</v>
       </c>
-      <c r="D27" s="8" t="s">
-        <v>584</v>
+      <c r="D27" s="8" t="str">
+        <v>Q107 approved; questionnaire reviewed. Draft/controls pending. Active: LEG-MT-032. PLAN.md §20.</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="15.75" customHeight="1">
@@ -12902,11 +12928,11 @@
       <c r="B28" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="C28" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D28" s="11" t="s">
-        <v>74</v>
+      <c r="C28" s="13" t="str">
+        <v>🔄 In Progress</v>
+      </c>
+      <c r="D28" s="11" t="str">
+        <v>Q96 approved; NCII questionnaire reviewed. Final policy, neutral review and controls pending. Active: LEG-MT-027. PLAN.md §20.</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="15.75" customHeight="1">
@@ -12933,8 +12959,8 @@
       <c r="C30" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D30" s="11" t="s">
-        <v>80</v>
+      <c r="D30" s="11" t="str">
+        <v>Q64 reporting direction approved; request-policy draft, NCMEC setup and evidence controls pending. PLAN.md §20.</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="15.75" customHeight="1">
@@ -12944,11 +12970,13 @@
       <c r="B31" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C31" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>83</v>
+      <c r="C31" s="91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">🔄 In Progress</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="str">
+        <v>Q122 approved; appeals questions reviewed. Final policy/controls pending. Active: LEG-MT-021. PLAN.md §20.</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="15.75" customHeight="1">
@@ -12958,11 +12986,13 @@
       <c r="B32" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="C32" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D32" s="11" t="s">
-        <v>86</v>
+      <c r="C32" s="91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">🔄 In Progress</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="str">
+        <v>Q114 approved; complaint questions reviewed. Final policy/controls pending. Active: LEG-MT-031. PLAN.md §20.</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="15.75" customHeight="1">
@@ -13100,17 +13130,17 @@
       </c>
     </row>
     <row r="43" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A43" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="B43" s="10" t="s">
-        <v>112</v>
+      <c r="A43" s="9" t="str">
+        <v>Define Founders recognition and benefits</v>
+      </c>
+      <c r="B43" s="10" t="str">
+        <v>Define Founders tag, Connect/Explore discovery and SFW events. Set eligibility, duration and prize terms.</v>
       </c>
       <c r="C43" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D43" s="11" t="s">
-        <v>113</v>
+      <c r="D43" s="11" t="str">
+        <v>Q132 approved Sept 22. Standard fees; no 500-person cap, member discount or permanent fee exemption. Q133 pending.</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="27.75" customHeight="1">
@@ -13329,14 +13359,14 @@
       <c r="A60" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="B60" s="6" t="s">
-        <v>146</v>
+      <c r="B60" s="6" t="str">
+        <v>Age eligibility and required verification before adult-content access; separate from content opt-in.</v>
       </c>
       <c r="C60" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D60" s="8" t="s">
-        <v>602</v>
+      <c r="D60" s="8" t="str">
+        <v>Q20: 18+ or higher legal minimum; location-based checks before adult access. Attestation exists; verification pending. PLAN.md §20.</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="24" customHeight="1">
@@ -13785,8 +13815,8 @@
       <c r="C94" s="91" t="s">
         <v>26</v>
       </c>
-      <c r="D94" s="11" t="s">
-        <v>619</v>
+      <c r="D94" s="11" t="str">
+        <v>Sales/site prep underway. Wallets deferred to future; direct pay stays. Processor approval and integration pending. PLAN.md §10.</v>
       </c>
     </row>
     <row r="95" spans="1:4" ht="15.75" customHeight="1">
@@ -13827,8 +13857,8 @@
       <c r="C97" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D97" s="11" t="s">
-        <v>622</v>
+      <c r="D97" s="11" t="str">
+        <v>Q23: self-service cancellation; paid-term access, refund exceptions and confirmation. Cutoff/setup pending. PLAN.md §20.</v>
       </c>
     </row>
     <row r="98" spans="1:4" ht="15.75" customHeight="1">
@@ -13855,8 +13885,8 @@
       <c r="C99" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D99" s="11" t="s">
-        <v>233</v>
+      <c r="D99" s="11" t="str">
+        <v>Q25: no unpaid pilot grace; retain paid access, pause at expiry until payment succeeds. Retry rules/setup pending. PLAN.md §20.</v>
       </c>
     </row>
     <row r="100" spans="1:4" ht="15.75" customHeight="1">
@@ -13883,14 +13913,14 @@
       <c r="A102" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="B102" s="6" t="s">
-        <v>238</v>
+      <c r="B102" s="6" t="str">
+        <v>Standard platform/creator split and calculation base. Founders use the same commission model.</v>
       </c>
       <c r="C102" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D102" s="11" t="s">
-        <v>623</v>
+      <c r="D102" s="11" t="str">
+        <v>Q131: 20/80 target; processing from platform share. Validate costs. Q132: standard fees for Founders.</v>
       </c>
     </row>
     <row r="103" spans="1:4" ht="15.75" customHeight="1">
@@ -13903,8 +13933,8 @@
       <c r="C103" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D103" s="11" t="s">
-        <v>624</v>
+      <c r="D103" s="11" t="str">
+        <v>Q28 approved: proportionate dispute handling; protect good-faith disputes. Review/build/tests pending. PLAN.md §20.</v>
       </c>
     </row>
     <row r="104" spans="1:4" ht="27.75" customHeight="1">
@@ -14048,25 +14078,25 @@
       <c r="D114" s="8"/>
     </row>
     <row r="115" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A115" s="9" t="s">
-        <v>262</v>
-      </c>
-      <c r="B115" s="10" t="s">
-        <v>263</v>
+      <c r="A115" s="9" t="str">
+        <v>Build Founders admin management</v>
+      </c>
+      <c r="B115" s="10" t="str">
+        <v>Manage Founders eligibility and badge assignment. Enforce a cohort limit only if approved.</v>
       </c>
       <c r="C115" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D115" s="11" t="s">
-        <v>264</v>
+      <c r="D115" s="11" t="str">
+        <v>Programme direction approved Q132; eligibility, cap and duration pending Q133. No implementation yet.</v>
       </c>
     </row>
     <row r="116" spans="1:4" ht="15.75" customHeight="1">
       <c r="A116" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="B116" s="6" t="s">
-        <v>266</v>
+      <c r="B116" s="6" t="str">
+        <v>Configure standard commission, content and feature flags, payout minimums and maintenance. No separate Founders rate.</v>
       </c>
       <c r="C116" s="13" t="s">
         <v>21</v>
@@ -14149,8 +14179,8 @@
       <c r="C122" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D122" s="8" t="s">
-        <v>281</v>
+      <c r="D122" s="8" t="str">
+        <v>Q16 daily urgent checks, including weekends; delegate when unavailable. Backup setup and workflow tests pending. PLAN.md §20.</v>
       </c>
     </row>
     <row r="123" spans="1:4" ht="15.75" customHeight="1">
@@ -14375,8 +14405,8 @@
       <c r="C139" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D139" s="11" t="s">
-        <v>323</v>
+      <c r="D139" s="11" t="str">
+        <v>Q18: no fixed date; CCBill timing unconfirmed. Limited pilot after approval and readiness checks. Checklist pending. PLAN.md §20.</v>
       </c>
     </row>
     <row r="140" spans="1:4" ht="15.75" customHeight="1">
@@ -14445,14 +14475,14 @@
       <c r="A146" s="9" t="s">
         <v>640</v>
       </c>
-      <c r="B146" s="10" t="s">
-        <v>641</v>
+      <c r="B146" s="10" t="str">
+        <v>Unlock individual creator content through approved hosted checkout, with ongoing access to the purchased version.</v>
       </c>
       <c r="C146" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D146" s="11" t="s">
-        <v>639</v>
+      <c r="D146" s="11" t="str">
+        <v>Q26: creator delisting preserves buyer access; legal/safety removals still apply. Paid flow pending. PLAN.md §20.</v>
       </c>
     </row>
     <row r="147" spans="1:4" ht="31.5" customHeight="1">
@@ -14549,8 +14579,8 @@
       <c r="C153" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D153" s="8" t="s">
-        <v>661</v>
+      <c r="D153" s="8" t="str">
+        <v>Q49: international pilot, separate role eligibility and active restrictions. Countries, budgets and implementation pending. PLAN.md §20.</v>
       </c>
     </row>
     <row r="154" spans="1:4" ht="15" customHeight="1">
@@ -14571,14 +14601,14 @@
       <c r="A155" s="5" t="s">
         <v>665</v>
       </c>
-      <c r="B155" s="6" t="s">
-        <v>666</v>
+      <c r="B155" s="6" t="str">
+        <v>Compare automated member age assurance and creator identity/age verification providers; preserve replaceable integration.</v>
       </c>
       <c r="C155" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D155" s="8" t="s">
-        <v>667</v>
+      <c r="D155" s="8" t="str">
+        <v>Sept 13: Ondato/Veriff candidates; provider, pricing and coverage unresolved. Coordinate CCBill review; no purchase approved. PLAN.md §20.</v>
       </c>
     </row>
     <row r="156" spans="1:4" ht="15" customHeight="1">
@@ -14605,8 +14635,8 @@
       <c r="C157" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D157" s="8" t="s">
-        <v>673</v>
+      <c r="D157" s="8" t="str">
+        <v>Sept 13 Q15 approved: Workspace Business aliases created; setup/tests pending. SES/Resend unselected. SMTP/Mailpit foundation only; production delivery pending. PLAN.md §20.</v>
       </c>
     </row>
     <row r="158" spans="1:4" ht="15" customHeight="1">
@@ -14627,14 +14657,14 @@
       <c r="A159" s="5" t="s">
         <v>677</v>
       </c>
-      <c r="B159" s="6" t="s">
-        <v>678</v>
+      <c r="B159" s="6" t="str">
+        <v>Validate processing, refunds, chargebacks, taxes, standard commission, payouts and programme costs. No Founders discount.</v>
       </c>
       <c r="C159" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D159" s="8" t="s">
-        <v>679</v>
+      <c r="D159" s="8" t="str">
+        <v>Q131: 20/80 target, actual economics pending. Q132: standard fees for Founders; cash-prize events need separate budgets.</v>
       </c>
     </row>
     <row r="160" spans="1:4" ht="36" customHeight="1">
@@ -21433,7 +21463,7 @@
       </c>
       <c r="E8" s="62">
         <f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A8,'Delivery Tracker'!$H$4:$H$400,"Done")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F8" s="62">
         <f>COUNTIF('Delivery Tracker'!$B$4:$B$400,$A8)</f>
@@ -21441,11 +21471,11 @@
       </c>
       <c r="G8" s="65">
         <f t="shared" si="0"/>
-        <v>0.14285714285714285</v>
+        <v>0.17142857142857143</v>
       </c>
       <c r="H8" s="62">
         <f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A8,'Delivery Tracker'!$H$4:$H$400,"In Progress")</f>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I8" s="62">
         <f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A8,'Delivery Tracker'!$H$4:$H$400,"In Review")</f>
@@ -21459,8 +21489,8 @@
         <f>COUNTIFS('Delivery Tracker'!$B$4:$B$400,$A8,'Delivery Tracker'!$H$4:$H$400,"Not Started")</f>
         <v>12</v>
       </c>
-      <c r="L8" s="62" t="s">
-        <v>901</v>
+      <c r="L8" t="str" s="62">
+        <v>Slices 1-4 published; operations dormant. Founder confirms Maryland approval and EIN receipt Sept 16. Legal review and business/provider dependencies remain open.</v>
       </c>
       <c r="M8" s="62" t="s">
         <v>902</v>
@@ -21471,8 +21501,8 @@
       <c r="O8" s="62" t="s">
         <v>904</v>
       </c>
-      <c r="P8" s="63">
-        <v>46271.666666666664</v>
+      <c r="P8" t="n" s="63">
+        <v>46281</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="57.95" customHeight="1">
@@ -23485,19 +23515,21 @@
         <v>814</v>
       </c>
       <c r="L27" s="62"/>
-      <c r="M27" s="62" t="s">
-        <v>970</v>
+      <c r="M27" s="62" t="str">
+        <v>Select SES/Resend for the hosted account flow after checking adult-business fit, cost and data handling; configure/test production delivery. PLAN.md §20.</v>
       </c>
       <c r="N27" s="63"/>
-      <c r="O27" s="62"/>
-      <c r="P27" s="63">
-        <v>46250.666666666664</v>
+      <c r="O27" s="62" t="str">
+        <v>Founder approval in chat, Sept 13; PLAN.md §20, Question 15.</v>
+      </c>
+      <c r="P27" s="63" t="n">
+        <v>46278</v>
       </c>
       <c r="Q27" s="62" t="s">
         <v>672</v>
       </c>
-      <c r="R27" s="62" t="s">
-        <v>673</v>
+      <c r="R27" s="62" t="str">
+        <v>Q15 approved. Workspace Business aliases created; setup/tests pending. SES/Resend unselected. SMTP/console and Mailpit implemented; production TLS, SPF/DKIM/DMARC, deliverability and bounce handling pending.</v>
       </c>
       <c r="S27" s="62" t="s">
         <v>1355</v>
@@ -24286,19 +24318,21 @@
         <v>808</v>
       </c>
       <c r="L42" s="62"/>
-      <c r="M42" s="62" t="s">
-        <v>974</v>
+      <c r="M42" s="62" t="str">
+        <v>Review approved answers in PLAN.md §20, including Q34's 60 days and Q35 venue exceptions. Obtain Q33 arbitration advice; finalize legal copy and live workflows. Plus deferred.</v>
       </c>
       <c r="N42" s="63"/>
-      <c r="O42" s="62"/>
-      <c r="P42" s="63">
-        <v>46250.666666666664</v>
+      <c r="O42" s="62" t="str">
+        <v>Founder approvals Sept 13–16; PLAN.md §20 Q21/Q27/Q30/Q32/Q33/Q34/Q35 and Plus note; apps/web/src/pages/RefundHelpPage.jsx (draft UI).</v>
+      </c>
+      <c r="P42" s="63" t="n">
+        <v>46281</v>
       </c>
       <c r="Q42" s="62" t="s">
         <v>25</v>
       </c>
-      <c r="R42" s="62" t="s">
-        <v>975</v>
+      <c r="R42" s="62" t="str">
+        <v>Suzanne's $1,100 bundle awaits review. Q34: 60 days; Q35: Maryland with rights exceptions. Q33 provider undecided. Plus deferred; refund UI draft. AUP/final notices and live workflows remain pending.</v>
       </c>
       <c r="S42" s="62" t="s">
         <v>976</v>
@@ -24337,19 +24371,21 @@
         <v>808</v>
       </c>
       <c r="L43" s="62"/>
-      <c r="M43" s="62" t="s">
-        <v>978</v>
+      <c r="M43" s="62" t="str">
+        <v>Apply Q50 to actual launch processing. Confirm Q51 vendor retention terms and implement Q46-48 controls after final review. Test mailbox routing and the restricted request log. PLAN.md §20.</v>
       </c>
       <c r="N43" s="63"/>
-      <c r="O43" s="62"/>
-      <c r="P43" s="63">
-        <v>46250.666666666664</v>
+      <c r="O43" s="62" t="str">
+        <v>Founder approval Sept 16, PLAN.md §20 Q50. EDPB territorial-scope and ICO transfer guidance linked there. Q51 pending retained.</v>
+      </c>
+      <c r="P43" s="63" t="n">
+        <v>46286</v>
       </c>
       <c r="Q43" s="62" t="s">
         <v>29</v>
       </c>
-      <c r="R43" s="62" t="s">
-        <v>30</v>
+      <c r="R43" s="62" t="str">
+        <v>Q50: draft for international creators/members. EU/UK provisions apply to covered processing, not nationality alone. Required controls precede processing. Vendor terms, implementation and review pending.</v>
       </c>
       <c r="S43" s="62" t="s">
         <v>979</v>
@@ -24378,8 +24414,8 @@
       <c r="H44" s="62" t="s">
         <v>529</v>
       </c>
-      <c r="I44" s="62" t="s">
-        <v>807</v>
+      <c r="I44" s="62" t="str">
+        <v>N/A</v>
       </c>
       <c r="J44" s="62" t="s">
         <v>368</v>
@@ -24388,19 +24424,21 @@
         <v>808</v>
       </c>
       <c r="L44" s="62"/>
-      <c r="M44" s="62" t="s">
-        <v>981</v>
+      <c r="M44" s="62" t="str">
+        <v>Finalize Community Rules from Q65-75 and implement enforcement before launch. Active founder review is under LEG-MT-015; no parallel founder task. PLAN.md §20.</v>
       </c>
       <c r="N44" s="63"/>
-      <c r="O44" s="62"/>
-      <c r="P44" s="63">
-        <v>46250.666666666664</v>
+      <c r="O44" s="62" t="str">
+        <v>Founder approval Sept 21, PLAN.md §20 Q75; Q74 retained as launch scope. Immediate-removal rules align with Q62-64, including review, preservation, notice and appeals.</v>
+      </c>
+      <c r="P44" s="63" t="n">
+        <v>46286</v>
       </c>
       <c r="Q44" s="62" t="s">
         <v>32</v>
       </c>
-      <c r="R44" s="62" t="s">
-        <v>33</v>
+      <c r="R44" s="62" t="str">
+        <v>Q75: substantiated serious violations may mean immediate termination; urgent removal/suspension pending review. Reports alone do not justify permanent bans. Final policy and controls pending.</v>
       </c>
       <c r="S44" s="62" t="s">
         <v>982</v>
@@ -24441,19 +24479,21 @@
       <c r="L45" s="62" t="s">
         <v>984</v>
       </c>
-      <c r="M45" s="62" t="s">
-        <v>985</v>
+      <c r="M45" s="62" t="str">
+        <v>Finalize AUP from Q53-64 decisions and review processor requirements; implement reporting, evidence preservation, moderation, notices and appeals before live use. Community review: LEG-MT-013.</v>
       </c>
       <c r="N45" s="63"/>
-      <c r="O45" s="62"/>
-      <c r="P45" s="63">
-        <v>46250.666666666664</v>
+      <c r="O45" s="62" t="str">
+        <v>Founder approval Sept 21, PLAN.md §20 Q64; 18 USC 2258A/2702 and NCMEC REPORT Act guidance. Prior content/enforcement decisions retained.</v>
+      </c>
+      <c r="P45" s="63" t="n">
+        <v>46286</v>
       </c>
       <c r="Q45" s="62" t="s">
         <v>35</v>
       </c>
-      <c r="R45" s="62" t="s">
-        <v>36</v>
+      <c r="R45" s="62" t="str">
+        <v>Q64: report apparent CSAM, child trafficking/enticement; emergency escalation and lawful disclosures. Secure evidence; covered CyberTipline material: one year from report. Setup/controls pending.</v>
       </c>
       <c r="S45" s="62" t="s">
         <v>986</v>
@@ -24482,8 +24522,8 @@
       <c r="H46" s="62" t="s">
         <v>529</v>
       </c>
-      <c r="I46" s="62" t="s">
-        <v>807</v>
+      <c r="I46" s="62" t="str">
+        <v>N/A</v>
       </c>
       <c r="J46" s="62" t="s">
         <v>368</v>
@@ -24492,19 +24532,21 @@
         <v>808</v>
       </c>
       <c r="L46" s="62"/>
-      <c r="M46" s="62" t="s">
-        <v>988</v>
+      <c r="M46" s="62" t="str">
+        <v>Finalize DMCA policy and case controls; complete contact setup, Q77 mail confirmation and registration before launch. Active founder review: LEG-MT-028. PLAN.md §20.</v>
       </c>
       <c r="N46" s="63"/>
-      <c r="O46" s="62"/>
-      <c r="P46" s="63">
-        <v>46250.666666666664</v>
+      <c r="O46" s="62" t="str">
+        <v>Founder approval Sept 21, PLAN.md §20 Q84-85: case-based enforcement, prompt notices and normal warnings; no fixed strike/warning allowance. Final policy and controls pending.</v>
+      </c>
+      <c r="P46" s="63" t="n">
+        <v>46286</v>
       </c>
       <c r="Q46" s="62" t="s">
         <v>38</v>
       </c>
-      <c r="R46" s="62" t="s">
-        <v>39</v>
+      <c r="R46" s="62" t="str">
+        <v>Founder: "Copyright Agent"; LLC provider; Pumdoki/pumdoki.com alternate names; dmca@pumdoki.com planned. Northwest phone selected; number/setup/testing and mail receipt unverified. Registration pending.</v>
       </c>
       <c r="S46" s="62" t="s">
         <v>989</v>
@@ -24543,19 +24585,21 @@
         <v>814</v>
       </c>
       <c r="L47" s="62"/>
-      <c r="M47" s="62" t="s">
-        <v>991</v>
+      <c r="M47" s="62" t="str">
+        <v>Confirm applicable duties and qualified custodian. Define segregated statutory records, separate consent storage, access and retention under Q38/Q46/Q55. Implement and review before live use.</v>
       </c>
       <c r="N47" s="63"/>
-      <c r="O47" s="62"/>
-      <c r="P47" s="63">
-        <v>46250.666666666664</v>
+      <c r="O47" s="62" t="str">
+        <v>Founder approval Sept 21, PLAN.md §20 Q55; Q38/Q46 retained. 28 CFR §75.2 and Mastercard §9.4.1.</v>
+      </c>
+      <c r="P47" s="63" t="n">
+        <v>46286</v>
       </c>
       <c r="Q47" s="62" t="s">
         <v>41</v>
       </c>
-      <c r="R47" s="62" t="s">
-        <v>42</v>
+      <c r="R47" s="62" t="str">
+        <v>Where §2257 applies, use a qualified custodian and segregate statutory records from consent files. One contracted provider may manage both. Producer duties remain; status/forms/provider not confirmed.</v>
       </c>
       <c r="S47" s="62" t="s">
         <v>992</v>
@@ -24753,21 +24797,21 @@
       <c r="L51" s="62" t="s">
         <v>997</v>
       </c>
-      <c r="M51" s="62" t="s">
-        <v>1004</v>
+      <c r="M51" s="62" t="str">
+        <v>Continue functioning-site/policy preparation. Apply current Mastercard adult rules and law; reconcile written CCBill/acquirer requirements before finalization.</v>
       </c>
       <c r="N51" s="63"/>
-      <c r="O51" s="62" t="s">
-        <v>1005</v>
-      </c>
-      <c r="P51" s="63">
-        <v>46275.666666666664</v>
+      <c r="O51" s="62" t="str">
+        <v>PLAN.md §20 Q17; docs/product/initial-ccbill-inquiry.md; Mastercard §9.4.1 (2026-08-04).</v>
+      </c>
+      <c r="P51" s="63" t="n">
+        <v>46278</v>
       </c>
       <c r="Q51" s="62" t="s">
         <v>53</v>
       </c>
-      <c r="R51" s="62" t="s">
-        <v>1006</v>
+      <c r="R51" s="62" t="str">
+        <v>Q17 approved. CCBill intake only; password-protected functioning site allowed. No detailed checklist/approval. Safe-content/R2 verified; policy drafting commissioned. Model, fees/reserves and payouts unresolved.</v>
       </c>
       <c r="S51" s="62" t="s">
         <v>1007</v>
@@ -24795,8 +24839,8 @@
       <c r="G52" s="62" t="s">
         <v>54</v>
       </c>
-      <c r="H52" s="62" t="s">
-        <v>532</v>
+      <c r="H52" s="62" t="str">
+        <v>In Progress</v>
       </c>
       <c r="I52" s="62" t="s">
         <v>836</v>
@@ -24807,22 +24851,24 @@
       <c r="K52" s="62" t="s">
         <v>808</v>
       </c>
-      <c r="L52" s="62" t="s">
-        <v>1010</v>
-      </c>
-      <c r="M52" s="62" t="s">
-        <v>970</v>
+      <c r="L52" s="62" t="str">
+        <v>Founder questionnaire review; commissioned draft pending</v>
+      </c>
+      <c r="M52" s="62" t="str">
+        <v>Review Q133 Founders duration and eligibility. Q132 benefits approved; exact placements and event/prize terms pending. PLAN.md §20.</v>
       </c>
       <c r="N52" s="63"/>
-      <c r="O52" s="62"/>
-      <c r="P52" s="63">
-        <v>46250.666666666664</v>
+      <c r="O52" s="62" t="str">
+        <v>Q132 approved Sept 22; Q133 pending. PLAN.md §20. Suzanne Lawyer bundle, Expense Tracker row 11; commissioned terms pending.</v>
+      </c>
+      <c r="P52" s="63" t="n">
+        <v>46287</v>
       </c>
       <c r="Q52" s="62" t="s">
         <v>55</v>
       </c>
-      <c r="R52" s="62" t="s">
-        <v>56</v>
+      <c r="R52" s="62" t="str">
+        <v>Q22: approval before creator publishing/monetization; applicable performer records before publication. Tax/payout documents before withdrawal or earlier if required. Forms/timing and implementation pending.</v>
       </c>
       <c r="S52" s="62" t="s">
         <v>1011</v>
@@ -25015,22 +25061,24 @@
       <c r="K56" s="62" t="s">
         <v>808</v>
       </c>
-      <c r="L56" s="62" t="s">
-        <v>1021</v>
-      </c>
-      <c r="M56" s="62" t="s">
-        <v>1022</v>
+      <c r="L56" t="str" s="62">
+        <v>Public-record check</v>
+      </c>
+      <c r="M56" t="str" s="62">
+        <v>Check the public Maryland record against the approved filing. Keep tax and internal ownership records private.</v>
       </c>
       <c r="N56" s="63"/>
-      <c r="O56" s="62"/>
-      <c r="P56" s="63">
-        <v>46273.666666666664</v>
+      <c r="O56" t="str" s="62">
+        <v>Founder reviewed initial filing, resolution and operating agreement and confirmed the name appears only in internal documents. Chat, September 16, 2026.</v>
+      </c>
+      <c r="P56" t="n" s="63">
+        <v>46281</v>
       </c>
       <c r="Q56" s="62" t="s">
         <v>66</v>
       </c>
-      <c r="R56" s="62" t="s">
-        <v>1023</v>
+      <c r="R56" t="str" s="62">
+        <v>Founder confirms state approval. Northwest address shown in dashboard; personal name absent from initial filing, present in internal resolution/agreement. Public SDAT record not independently checked.</v>
       </c>
       <c r="S56" s="62" t="s">
         <v>1024</v>
@@ -25068,18 +25116,18 @@
       <c r="K57" s="62" t="s">
         <v>808</v>
       </c>
-      <c r="L57" s="62" t="s">
-        <v>997</v>
-      </c>
-      <c r="M57" s="62" t="s">
-        <v>1028</v>
+      <c r="L57" s="62" t="str">
+        <v>Commissioned draft and substantive review pending</v>
+      </c>
+      <c r="M57" s="62" t="str">
+        <v>Review commissioned policy; assess specialist participation and processor requirements; implement/test controls. Active founder review: LEG-MT-032. PLAN.md §20.</v>
       </c>
       <c r="N57" s="63"/>
-      <c r="O57" s="62" t="s">
-        <v>1029</v>
-      </c>
-      <c r="P57" s="63">
-        <v>46275.666666666664</v>
+      <c r="O57" s="62" t="str">
+        <v>Q107 approved Sept 22; questionnaire reviewed. PLAN.md §20. Suzanne Lawyer $1,100 bundle recorded in Expense Tracker row 11; draft and controls pending.</v>
+      </c>
+      <c r="P57" s="63" t="n">
+        <v>46287</v>
       </c>
       <c r="Q57" s="62" t="s">
         <v>71</v>
@@ -25111,8 +25159,8 @@
       <c r="G58" s="62" t="s">
         <v>72</v>
       </c>
-      <c r="H58" s="62" t="s">
-        <v>532</v>
+      <c r="H58" s="62" t="str">
+        <v>In Progress</v>
       </c>
       <c r="I58" s="62" t="s">
         <v>836</v>
@@ -25123,16 +25171,18 @@
       <c r="K58" s="62" t="s">
         <v>808</v>
       </c>
-      <c r="L58" s="62" t="s">
-        <v>997</v>
-      </c>
-      <c r="M58" s="62" t="s">
-        <v>970</v>
+      <c r="L58" s="62" t="str">
+        <v>Final policy and controls pending</v>
+      </c>
+      <c r="M58" s="62" t="str">
+        <v>Finalize policy, retention periods and applicable neutral-review arrangements; implement/test NCII controls. Active founder review: LEG-MT-027. PLAN.md §20.</v>
       </c>
       <c r="N58" s="63"/>
-      <c r="O58" s="62"/>
-      <c r="P58" s="63">
-        <v>46250.666666666664</v>
+      <c r="O58" s="62" t="str">
+        <v>Founder approval Sept 21, PLAN.md §20 Q96: human appeals, consent-based restoration and applicable neutral review at Pumdoki expense. Provider/controls pending.</v>
+      </c>
+      <c r="P58" s="63" t="n">
+        <v>46286</v>
       </c>
       <c r="Q58" s="62" t="s">
         <v>73</v>
@@ -25230,19 +25280,21 @@
       <c r="L60" s="62" t="s">
         <v>984</v>
       </c>
-      <c r="M60" s="62" t="s">
-        <v>970</v>
+      <c r="M60" s="62" t="str">
+        <v>Draft government-request handling using Q64 reporting/preservation boundaries. Define lawful disclosures, notices, emergency contacts, NCMEC setup and restricted evidence procedures before live use.</v>
       </c>
       <c r="N60" s="63"/>
-      <c r="O60" s="62"/>
-      <c r="P60" s="63">
-        <v>46250.666666666664</v>
+      <c r="O60" s="62" t="str">
+        <v>Founder approval Sept 21, PLAN.md §20 Q64; 18 USC 2258A/2702. Reporting direction recorded; full government-request policy remains undrafted.</v>
+      </c>
+      <c r="P60" s="63" t="n">
+        <v>46286</v>
       </c>
       <c r="Q60" s="62" t="s">
         <v>79</v>
       </c>
-      <c r="R60" s="62" t="s">
-        <v>80</v>
+      <c r="R60" s="62" t="str">
+        <v>Q64: mandatory CyberTipline reports, urgent emergency escalation, lawful referrals/disclosures, secure preservation. Covered report material: one year; longer if required. Full policy/controls pending.</v>
       </c>
       <c r="S60" s="62" t="s">
         <v>1037</v>
@@ -25268,8 +25320,8 @@
       <c r="G61" s="62" t="s">
         <v>81</v>
       </c>
-      <c r="H61" s="62" t="s">
-        <v>532</v>
+      <c r="H61" s="62" t="str">
+        <v>In Progress</v>
       </c>
       <c r="I61" s="62" t="s">
         <v>836</v>
@@ -25280,20 +25332,24 @@
       <c r="K61" s="62" t="s">
         <v>808</v>
       </c>
-      <c r="L61" s="62"/>
-      <c r="M61" s="62" t="s">
-        <v>970</v>
+      <c r="L61" s="62" t="str">
+        <v>Commissioned draft and substantive review pending</v>
+      </c>
+      <c r="M61" s="62" t="str">
+        <v>Review commissioned policy; implement/test appeals, notices, external review and financial corrections. Active founder review: LEG-MT-021. PLAN.md §20.</v>
       </c>
       <c r="N61" s="63"/>
-      <c r="O61" s="62"/>
-      <c r="P61" s="63">
-        <v>46250.666666666664</v>
+      <c r="O61" s="62" t="str">
+        <v>Q122 approved Sept 22; appeals questions reviewed. PLAN.md §20. Suzanne Lawyer bundle, Expense Tracker row 11; final policy and controls pending.</v>
+      </c>
+      <c r="P61" s="63" t="n">
+        <v>46287</v>
       </c>
       <c r="Q61" s="62" t="s">
         <v>82</v>
       </c>
-      <c r="R61" s="62" t="s">
-        <v>83</v>
+      <c r="R61" s="62" t="str">
+        <v>Drafting commissioned in purchased bundle. Final review, applicable neutral-review arrangements and appeal controls pending before creator onboarding.</v>
       </c>
       <c r="S61" s="62" t="s">
         <v>1039</v>
@@ -25319,8 +25375,8 @@
       <c r="G62" s="62" t="s">
         <v>84</v>
       </c>
-      <c r="H62" s="62" t="s">
-        <v>532</v>
+      <c r="H62" s="62" t="str">
+        <v>In Progress</v>
       </c>
       <c r="I62" s="62" t="s">
         <v>836</v>
@@ -25331,20 +25387,24 @@
       <c r="K62" s="62" t="s">
         <v>808</v>
       </c>
-      <c r="L62" s="62"/>
-      <c r="M62" s="62" t="s">
-        <v>970</v>
+      <c r="L62" s="62" t="str">
+        <v>Commissioned draft and substantive review pending</v>
+      </c>
+      <c r="M62" s="62" t="str">
+        <v>Review commissioned policy and implement/test intake, case tracking, deadlines and backup coverage. Active founder review: LEG-MT-031. PLAN.md §20.</v>
       </c>
       <c r="N62" s="63"/>
-      <c r="O62" s="62"/>
-      <c r="P62" s="63">
-        <v>46250.666666666664</v>
+      <c r="O62" s="62" t="str">
+        <v>Q114 approved Sept 22; complaint questions reviewed. PLAN.md §20. Complaints/appeals drafting in Suzanne Lawyer bundle (Expense Tracker row 11); delivery/approval pending.</v>
+      </c>
+      <c r="P62" s="63" t="n">
+        <v>46287</v>
       </c>
       <c r="Q62" s="62" t="s">
         <v>85</v>
       </c>
-      <c r="R62" s="62" t="s">
-        <v>86</v>
+      <c r="R62" s="62" t="str">
+        <v>Q7 aliases created; routing/tests pending. Q16/Q98 backup and urgent coverage planned. Drafting purchased; final policy and 7-business-day/48-hour controls pending.</v>
       </c>
       <c r="S62" s="62" t="s">
         <v>1041</v>
@@ -25548,29 +25608,21 @@
           <t xml:space="preserve">Launch-country rules + provider/privacy review</t>
         </is>
       </c>
-      <c r="M66" s="62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Define country triggers with LEG-MT-153; select a provider and retention rules. Then implement and test the age gate before live adult access.</t>
-        </is>
+      <c r="M66" s="62" t="str">
+        <v>Finalize location/risk triggers with LEG-MT-153 and provider/data handling with LEG-MT-155; implement/test required server-side checks before live adult access.</v>
       </c>
       <c r="N66" s="63"/>
-      <c r="O66" s="62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://help.fansly.com/en/articles/11845000-global-age-verification-requirement</t>
-        </is>
-      </c>
-      <c r="P66" s="63">
-        <v>46275</v>
-      </c>
-      <c r="Q66" s="62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jurisdiction-aware 18+ verification before restricted adult content: login/content-entry prompt, provider-hosted selfie/liveness check and ID fallback if required, persisted verified status, and retry/help states. Enforce required checks server-side. Keep this separate from content opt-in and creator identity/performer records.</t>
-        </is>
-      </c>
-      <c r="R66" s="62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Registration records append-only age attestation and versioned Terms/Privacy acceptance; verified email gates creator-application submission. Entry-gate UI and actual identity/age verification remain pending. September 10: global flow added to scope; implementation not started. Fansly reference reviewed; its provider, country list, timing and retention claims are not adopted. Review actual coverage/data handling before live use.</t>
-        </is>
+      <c r="O66" s="62" t="str">
+        <v>PLAN.md §3.5/§20 Q20; founder approval Sept 13; https://help.fansly.com/en/articles/11845000-global-age-verification-requirement</v>
+      </c>
+      <c r="P66" s="63" t="n">
+        <v>46278</v>
+      </c>
+      <c r="Q66" s="62" t="str">
+        <v>18+ or higher legal minimum. Member checks follow jurisdiction/law, processor requirements and risk controls. Login/content-entry prompt; provider-hosted selfie/liveness and ID fallback if required; saved status and retry/help states. Enforce required checks server-side before adult access. Separate from content opt-in and creator identity/performer records.</v>
+      </c>
+      <c r="R66" s="62" t="str">
+        <v>Q20 approved. Age attestation and Terms/Privacy evidence exist; verified email gates creator applications. Required age checks cannot be replaced by attestation. Provider, country rules and verification setup/tests pending. Fansly details are not adopted.</v>
       </c>
       <c r="S66" s="62" t="s">
         <v>1115</v>
@@ -25664,19 +25716,21 @@
       <c r="L68" s="62" t="s">
         <v>1010</v>
       </c>
-      <c r="M68" s="62" t="s">
-        <v>970</v>
+      <c r="M68" s="62" t="str">
+        <v>Before pilot: confirm creator/member country lists, member cap, verification budget and cash buffer. Implement/test Q49 access restrictions. Creator tax forms: LEG-MT-021.</v>
       </c>
       <c r="N68" s="63"/>
-      <c r="O68" s="62"/>
-      <c r="P68" s="63">
-        <v>46250.666666666664</v>
+      <c r="O68" s="62" t="str">
+        <v>Founder approvals Sept 13 and 16. PLAN.md §3.6 and §20, Q9-10 and Q49. Published eligibility/age-check comparison sources linked there.</v>
+      </c>
+      <c r="P68" s="63" t="n">
+        <v>46281</v>
       </c>
       <c r="Q68" s="62" t="s">
         <v>660</v>
       </c>
-      <c r="R68" s="62" t="s">
-        <v>661</v>
+      <c r="R68" s="62" t="str">
+        <v>Q49 approved: broad international objective, separate creator/member eligibility, active restrictions and required age checks before adult access. Country lists, budgets, providers and controls pending.</v>
       </c>
       <c r="S68" s="62" t="s">
         <v>1346</v>
@@ -25770,19 +25824,21 @@
         <v>814</v>
       </c>
       <c r="L70" s="62"/>
-      <c r="M70" s="62" t="s">
-        <v>970</v>
+      <c r="M70" s="62" t="str">
+        <v>Compare Ondato/Veriff coverage, total pilot cost and privacy/retention terms; coordinate CCBill review requirements before selection.</v>
       </c>
       <c r="N70" s="63"/>
-      <c r="O70" s="62"/>
-      <c r="P70" s="63">
-        <v>46250.666666666664</v>
-      </c>
-      <c r="Q70" s="62" t="s">
-        <v>666</v>
-      </c>
-      <c r="R70" s="62" t="s">
-        <v>667</v>
+      <c r="O70" s="62" t="str">
+        <v>Founder approval in chat, Sept 13; PLAN.md §3.5 and §20, Question 12.</v>
+      </c>
+      <c r="P70" s="63" t="n">
+        <v>46278</v>
+      </c>
+      <c r="Q70" s="62" t="str">
+        <v>Compare automated member age assurance and creator identity/age verification providers; preserve replaceable integration.</v>
+      </c>
+      <c r="R70" s="62" t="str">
+        <v>Sept 13: Ondato/Veriff candidates; no provider selected. Automated flows planned; configure/test before live adult access or real creator identity onboarding. No purchase or fixed CCBill deadline approved.</v>
       </c>
       <c r="S70" s="62" t="s">
         <v>1351</v>
@@ -25808,8 +25864,8 @@
       <c r="G71" s="62" t="s">
         <v>1357</v>
       </c>
-      <c r="H71" s="62" t="s">
-        <v>529</v>
+      <c r="H71" t="str" s="62">
+        <v>Done</v>
       </c>
       <c r="I71" s="62" t="s">
         <v>836</v>
@@ -25820,22 +25876,22 @@
       <c r="K71" s="62" t="s">
         <v>808</v>
       </c>
-      <c r="L71" s="62" t="s">
-        <v>1358</v>
-      </c>
-      <c r="M71" s="62" t="s">
-        <v>1359</v>
+      <c r="L71" s="62"/>
+      <c r="M71" t="str" s="62">
+        <v>Retain state approval and IRS confirmation privately. Banking and DBA registration remain separate follow-ups.</v>
       </c>
       <c r="N71" s="63"/>
-      <c r="O71" s="62"/>
-      <c r="P71" s="63">
-        <v>46273.666666666664</v>
-      </c>
-      <c r="Q71" s="62" t="s">
-        <v>1360</v>
-      </c>
-      <c r="R71" s="62" t="s">
-        <v>1361</v>
+      <c r="O71" t="str" s="62">
+        <v>Founder confirmed Maryland approval and supplied the issued EIN in chat on September 16, 2026. PLAN.md section 20.</v>
+      </c>
+      <c r="P71" t="n" s="63">
+        <v>46281</v>
+      </c>
+      <c r="Q71" t="str" s="62">
+        <v>Kiban Digital Holdings LLC: Maryland formation approved and EIN obtained, confirmed by the founder September 16, 2026.</v>
+      </c>
+      <c r="R71" t="str" s="62">
+        <v>Filed through Northwest. Founder confirmed approval and EIN receipt Sept 16. Original state/IRS documents not independently inspected; EIN held outside Git. Banking/DBA remain open.</v>
       </c>
       <c r="S71" s="62" t="s">
         <v>1362</v>
@@ -26667,8 +26723,8 @@
       <c r="F87" s="62" t="s">
         <v>1069</v>
       </c>
-      <c r="G87" s="62" t="s">
-        <v>111</v>
+      <c r="G87" s="62" t="str">
+        <v>Define Founders recognition and benefits</v>
       </c>
       <c r="H87" s="62" t="s">
         <v>532</v>
@@ -26683,19 +26739,21 @@
         <v>814</v>
       </c>
       <c r="L87" s="62"/>
-      <c r="M87" s="62" t="s">
-        <v>1070</v>
+      <c r="M87" s="62" t="str">
+        <v>Define eligibility and duration after Q133. Plan Founders tag, Connect filter or Explore section, SFW Discord events and future event priority.</v>
       </c>
       <c r="N87" s="63"/>
-      <c r="O87" s="62"/>
-      <c r="P87" s="63">
-        <v>46271.666666666664</v>
-      </c>
-      <c r="Q87" s="62" t="s">
-        <v>112</v>
-      </c>
-      <c r="R87" s="62" t="s">
-        <v>1071</v>
+      <c r="O87" s="62" t="str">
+        <v>Q132 approved Sept 22. PLAN.md §20 supersedes commission-free/cost-recovery terms; Q133 pending.</v>
+      </c>
+      <c r="P87" s="63" t="n">
+        <v>46287</v>
+      </c>
+      <c r="Q87" s="62" t="str">
+        <v>Founders tag; Connect filter or Explore section below top sections; SFW Discord events; future event priority. No special commission.</v>
+      </c>
+      <c r="R87" s="62" t="str">
+        <v>No fixed cohort, permanent ranking, member discount or Plus promise. Cash prizes optional and separately budgeted. Implementation not started.</v>
       </c>
       <c r="S87" s="62" t="s">
         <v>1072</v>
@@ -26838,21 +26896,21 @@
       <c r="L90" s="62" t="s">
         <v>997</v>
       </c>
-      <c r="M90" s="62" t="s">
-        <v>1206</v>
+      <c r="M90" s="62" t="str">
+        <v>Continue the functioning review site. Return to CCBill when review-ready; confirm direct-payment terms before integration. Wallet assessment/build are future work. PLAN.md §20.</v>
       </c>
       <c r="N90" s="63"/>
-      <c r="O90" s="62" t="s">
-        <v>1207</v>
-      </c>
-      <c r="P90" s="63">
-        <v>46275.666666666664</v>
+      <c r="O90" s="62" t="str">
+        <v>Initial CCBill inquiry record; Sept 13 final wallet deferral; PLAN.md Phase 6/§20 and HANDOFF.md.</v>
+      </c>
+      <c r="P90" s="63" t="n">
+        <v>46278</v>
       </c>
       <c r="Q90" s="62" t="s">
         <v>1208</v>
       </c>
-      <c r="R90" s="62" t="s">
-        <v>1209</v>
+      <c r="R90" s="62" t="str">
+        <v>Sales replied; functioning site required. Founder deferred wallets to future and resumed questionnaire. Candidate preserved; no active wallet assessment/build. Provider approval and payment backend pending.</v>
       </c>
       <c r="S90" s="62" t="s">
         <v>1210</v>
@@ -26999,19 +27057,21 @@
       <c r="L93" s="62" t="s">
         <v>997</v>
       </c>
-      <c r="M93" s="62" t="s">
-        <v>1220</v>
+      <c r="M93" s="62" t="str">
+        <v>Confirm processor-supported billing/cancellation flow, cutoff and account setup; implement trusted events and test cancellation, expiry and confirmation. PLAN.md §20 Q23.</v>
       </c>
       <c r="N93" s="63"/>
-      <c r="O93" s="62"/>
-      <c r="P93" s="63">
-        <v>46275.666666666664</v>
+      <c r="O93" s="62" t="str">
+        <v>Founder approval Sept 13; PLAN.md §20 Q23 and cited Fansly/CCBill sources.</v>
+      </c>
+      <c r="P93" s="63" t="n">
+        <v>46278</v>
       </c>
       <c r="Q93" s="62" t="s">
         <v>227</v>
       </c>
-      <c r="R93" s="62" t="s">
-        <v>1221</v>
+      <c r="R93" s="62" t="str">
+        <v>CCBill review-site preparation underway. Q23 cancellation approved: paid-term access, refund exceptions and confirmation. Cutoff unconfirmed; recurring billing, webhooks and cancellation remain unimplemented.</v>
       </c>
       <c r="S93" s="62" t="s">
         <v>1222</v>
@@ -27101,19 +27161,21 @@
         <v>814</v>
       </c>
       <c r="L95" s="62"/>
-      <c r="M95" s="62" t="s">
-        <v>970</v>
+      <c r="M95" s="62" t="str">
+        <v>Confirm processor retry/expiry semantics; implement trusted paid-through access and recovery after payment. Test that failure does not revoke other purchases. PLAN.md §20 Q25.</v>
       </c>
       <c r="N95" s="63"/>
-      <c r="O95" s="62"/>
-      <c r="P95" s="63">
-        <v>46250.666666666664</v>
+      <c r="O95" s="62" t="str">
+        <v>Founder approval Sept 13; PLAN.md §20 Q25 and cited CCBill event documentation.</v>
+      </c>
+      <c r="P95" s="63" t="n">
+        <v>46278</v>
       </c>
       <c r="Q95" s="62" t="s">
         <v>232</v>
       </c>
-      <c r="R95" s="62" t="s">
-        <v>233</v>
+      <c r="R95" s="62" t="str">
+        <v>Q25 approved: no automatic unpaid pilot grace. Retain paid access; pause affected subscription at expiry until payment confirmed. No whole-account suspension or loss of other purchases. Retry/status details pending.</v>
       </c>
       <c r="S95" s="62" t="s">
         <v>1226</v>
@@ -27207,19 +27269,21 @@
       <c r="L97" s="62" t="s">
         <v>997</v>
       </c>
-      <c r="M97" s="62" t="s">
-        <v>970</v>
+      <c r="M97" s="62" t="str">
+        <v>Validate Q131 20/80 target against actual provider and operating costs. Founders use standard commission. Final commercial terms pending.</v>
       </c>
       <c r="N97" s="63"/>
-      <c r="O97" s="62"/>
-      <c r="P97" s="63">
-        <v>46250.666666666664</v>
-      </c>
-      <c r="Q97" s="62" t="s">
-        <v>238</v>
-      </c>
-      <c r="R97" s="62" t="s">
-        <v>623</v>
+      <c r="O97" s="62" t="str">
+        <v>Q131–132 approved Sept 22. PLAN.md §3.8 and §20. No provider quote or live payment approval.</v>
+      </c>
+      <c r="P97" s="63" t="n">
+        <v>46287</v>
+      </c>
+      <c r="Q97" s="62" t="str">
+        <v>20% platform / 80% creator target excluding sales tax/VAT; ordinary processing costs from platform share. Same commission for Founders.</v>
+      </c>
+      <c r="R97" s="62" t="str">
+        <v>Validate sustainability before a firm offer or live payments. Refund/chargeback allocation, payout fees and paid-session commission pending.</v>
       </c>
       <c r="S97" s="62" t="s">
         <v>1230</v>
@@ -27260,19 +27324,21 @@
       <c r="L98" s="62" t="s">
         <v>997</v>
       </c>
-      <c r="M98" s="62" t="s">
-        <v>1232</v>
+      <c r="M98" s="62" t="str">
+        <v>Review Q28 with counsel/processor; define trusted dispute events, then implement and test transaction access, proportionate restrictions, authorized operations and audit. PLAN.md §20.</v>
       </c>
       <c r="N98" s="63"/>
-      <c r="O98" s="62"/>
-      <c r="P98" s="63">
-        <v>46275.666666666664</v>
+      <c r="O98" s="62" t="str">
+        <v>Founder approval Sept 14, 2026; PLAN.md §20 Q28; CFPB dispute guidance and Fansly/LoyalFans policy references recorded there.</v>
+      </c>
+      <c r="P98" s="63" t="n">
+        <v>46279</v>
       </c>
       <c r="Q98" s="62" t="s">
         <v>240</v>
       </c>
-      <c r="R98" s="62" t="s">
-        <v>1233</v>
+      <c r="R98" s="62" t="str">
+        <v>Q28: review disputed access; keep unrelated valid purchases. No penalty solely for good-faith disputes. Broader restrictions need justification. Legal/processor review, integration and handling pending.</v>
       </c>
       <c r="S98" s="62" t="s">
         <v>1234</v>
@@ -27362,19 +27428,21 @@
         <v>814</v>
       </c>
       <c r="L100" s="62"/>
-      <c r="M100" s="62" t="s">
-        <v>1322</v>
+      <c r="M100" s="62" t="str">
+        <v>Confirm processor terms; implement hosted checkout, verified payment, retained purchased versions and buyer access after creator delisting. Test required removals separately. PLAN.md §20 Q26.</v>
       </c>
       <c r="N100" s="63"/>
-      <c r="O100" s="62"/>
-      <c r="P100" s="63">
-        <v>46274.666666666664</v>
-      </c>
-      <c r="Q100" s="62" t="s">
-        <v>1323</v>
-      </c>
-      <c r="R100" s="62" t="s">
-        <v>1324</v>
+      <c r="O100" s="62" t="str">
+        <v>Founder approval Sept 13; PLAN.md §20 Q26 and cited Fansly sold-media guidance.</v>
+      </c>
+      <c r="P100" s="63" t="n">
+        <v>46278</v>
+      </c>
+      <c r="Q100" s="62" t="str">
+        <v>One-off hosted checkout for individual photos/videos or bundles; verified payment grants ongoing access to the purchased version. Ordinary creator delisting preserves buyer access.</v>
+      </c>
+      <c r="R100" s="62" t="str">
+        <v>Q26 approved: no scheduled purchase expiry. Retain media and buyer grants after ordinary delisting; legal/safety removals and Terms/Refund Policy still apply. Processor approval and paid flow remain pending.</v>
       </c>
       <c r="S100" s="62" t="s">
         <v>1325</v>
@@ -27415,19 +27483,21 @@
       <c r="L101" s="62" t="s">
         <v>997</v>
       </c>
-      <c r="M101" s="62" t="s">
-        <v>970</v>
+      <c r="M101" s="62" t="str">
+        <v>Model actual processing, taxes, refunds, chargebacks, payout timing and operating costs against Q131. Include optional Founders event budgets.</v>
       </c>
       <c r="N101" s="63"/>
-      <c r="O101" s="62"/>
-      <c r="P101" s="63">
-        <v>46250.666666666664</v>
-      </c>
-      <c r="Q101" s="62" t="s">
-        <v>678</v>
-      </c>
-      <c r="R101" s="62" t="s">
-        <v>679</v>
+      <c r="O101" s="62" t="str">
+        <v>Q131/Q132 approved. See PLAN.md section 20.</v>
+      </c>
+      <c r="P101" s="63" t="n">
+        <v>46287</v>
+      </c>
+      <c r="Q101" s="62" t="str">
+        <v>Validate standard commission and payout economics, including programme costs. No Founders discount or commission exemption.</v>
+      </c>
+      <c r="R101" s="62" t="str">
+        <v>20/80 is an approved target, not proven profitability. Prize amounts and recurring event spend are not approved.</v>
       </c>
       <c r="S101" s="62" t="s">
         <v>1364</v>
@@ -28753,8 +28823,8 @@
       <c r="F127" s="62" t="s">
         <v>1202</v>
       </c>
-      <c r="G127" s="62" t="s">
-        <v>262</v>
+      <c r="G127" s="62" t="str">
+        <v>Build Founders admin management</v>
       </c>
       <c r="H127" s="62" t="s">
         <v>532</v>
@@ -28771,19 +28841,19 @@
       <c r="L127" s="62" t="s">
         <v>1203</v>
       </c>
-      <c r="M127" s="62" t="s">
-        <v>970</v>
+      <c r="M127" s="62" t="str">
+        <v>After Q133 terms and private-operations gates, implement Founders eligibility and badge management. No fixed cohort cap assumed.</v>
       </c>
       <c r="N127" s="63"/>
       <c r="O127" s="62"/>
-      <c r="P127" s="63">
-        <v>46250.666666666664</v>
-      </c>
-      <c r="Q127" s="62" t="s">
-        <v>263</v>
-      </c>
-      <c r="R127" s="62" t="s">
-        <v>264</v>
+      <c r="P127" s="63" t="n">
+        <v>46287</v>
+      </c>
+      <c r="Q127" s="62" t="str">
+        <v>Manage Founders eligibility and badge assignment. Enforce a cohort limit only if approved.</v>
+      </c>
+      <c r="R127" s="62" t="str">
+        <v>Q132 programme direction approved; Q133 eligibility/duration pending. No member discount or separate Founders rate.</v>
       </c>
       <c r="S127" s="62" t="s">
         <v>1260</v>
@@ -28829,11 +28899,11 @@
       </c>
       <c r="N128" s="63"/>
       <c r="O128" s="62"/>
-      <c r="P128" s="63">
-        <v>46250.666666666664</v>
-      </c>
-      <c r="Q128" s="62" t="s">
-        <v>266</v>
+      <c r="P128" s="63" t="n">
+        <v>46287</v>
+      </c>
+      <c r="Q128" s="62" t="str">
+        <v>Configure standard commission, content/feature flags, payout minimums and maintenance. No separate Founders commission setting.</v>
       </c>
       <c r="R128" s="62" t="s">
         <v>267</v>
@@ -29456,19 +29526,21 @@
         <v>814</v>
       </c>
       <c r="L140" s="62"/>
-      <c r="M140" s="62" t="s">
-        <v>970</v>
+      <c r="M140" s="62" t="str">
+        <v>Configure email intake, receipts, urgent alerts and deadline tracking; arrange backup coverage and test before live use. PLAN.md §20, Q16.</v>
       </c>
       <c r="N140" s="63"/>
-      <c r="O140" s="62"/>
-      <c r="P140" s="63">
-        <v>46250.666666666664</v>
+      <c r="O140" s="62" t="str">
+        <v>Founder confirmation in chat, Sept 13; PLAN.md §20, Question 16.</v>
+      </c>
+      <c r="P140" s="63" t="n">
+        <v>46278</v>
       </c>
       <c r="Q140" s="62" t="s">
         <v>280</v>
       </c>
-      <c r="R140" s="62" t="s">
-        <v>281</v>
+      <c r="R140" s="62" t="str">
+        <v>Q16: founder email support; daily urgent checks including weekends; delegate when unavailable. No backup assigned. Routine human reply target: 2 business days. Complaint/NCII deadlines: PLAN.md §20.</v>
       </c>
       <c r="S140" s="62" t="s">
         <v>1272</v>
@@ -30180,19 +30252,21 @@
         <v>814</v>
       </c>
       <c r="L154" s="62"/>
-      <c r="M154" s="62" t="s">
-        <v>970</v>
+      <c r="M154" s="62" t="str">
+        <v>Define and verify limited-pilot readiness criteria alongside functional slices: processor approval plus product, legal, safety, security and support checks.</v>
       </c>
       <c r="N154" s="63"/>
-      <c r="O154" s="62"/>
-      <c r="P154" s="63">
-        <v>46250.666666666664</v>
+      <c r="O154" s="62" t="str">
+        <v>Founder approval, Sept 13; PLAN.md §20 Q18; docs/product/initial-ccbill-inquiry.md.</v>
+      </c>
+      <c r="P154" s="63" t="n">
+        <v>46278</v>
       </c>
       <c r="Q154" s="62" t="s">
         <v>322</v>
       </c>
-      <c r="R154" s="62" t="s">
-        <v>323</v>
+      <c r="R154" s="62" t="str">
+        <v>Q18 approved: no fixed date or confirmed underwriting duration. Limited member pilot after approval/checks; expansion depends on results, country coverage and capacity. Checklist remains incomplete.</v>
       </c>
       <c r="S154" s="62" t="s">
         <v>1311</v>

</xml_diff>

<commit_message>
feat: add refund help and finalize questionnaire handoff
</commit_message>
<xml_diff>
--- a/docs/product/Pumdoki_MasterTracker_V4.xlsx
+++ b/docs/product/Pumdoki_MasterTracker_V4.xlsx
@@ -11210,10 +11210,10 @@
         <v>Q131 approves a 20/80 target excluding sales tax; processing costs from platform share. Q132 applies standard fees to Founders, replacing cost-recovery terms.</v>
       </c>
       <c r="H14" s="62" t="str">
-        <v>Validate actual costs before firm pricing/live payments. Refund/chargeback allocation and payout fees pending. Budget prize events separately.</v>
+        <v>Validate actual costs under Q139–141 loss/fee rules. Provider payout fees remain unconfirmed. Budget prize events separately.</v>
       </c>
       <c r="I14" s="62" t="str">
-        <v>PLAN.md §3.8 and §20, Q131–132 approved September 22, 2026.</v>
+        <v>PLAN.md §§3.8,20: Q131–132 and Q139–141 approved September 22, 2026.</v>
       </c>
       <c r="J14" s="63" t="n">
         <v>46287</v>
@@ -11484,10 +11484,10 @@
         <v>Q132: Founders tag; Connect filter or Explore section below top sections; SFW Discord events; future event priority. Standard fees replace commission exemption.</v>
       </c>
       <c r="H23" s="69" t="str">
-        <v>Q133: define eligibility, cutoff/cap and duration. Specify placements and event terms; cash prizes optional, separately funded. No sales/ranking guarantee.</v>
+        <v>Q133: tag lasts for eligible account life; discovery/event priority conditional. Finalize eligibility, cutoff/cap and event terms; fund prizes separately.</v>
       </c>
       <c r="I23" s="69" t="str">
-        <v>PLAN.md §20, Q132 approved September 22, 2026; Q133 pending.</v>
+        <v>PLAN.md §20, Q132–133 approved September 22, 2026; eligibility and event details remain open.</v>
       </c>
       <c r="J23" s="70" t="n">
         <v>46287</v>
@@ -12834,7 +12834,7 @@
         <v>🔄 In Progress</v>
       </c>
       <c r="D21" s="8" t="str">
-        <v>Q132 approved: Founders benefits replace fee exemption. Review Q133 duration and eligibility. PLAN.md §20.</v>
+        <v>Final questionnaire corrections confirmed by founder. Await Suzanne response and drafts; provider/legal review pending. PLAN §20.</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="15.75" customHeight="1">
@@ -13140,7 +13140,7 @@
         <v>21</v>
       </c>
       <c r="D43" s="11" t="str">
-        <v>Q132 approved Sept 22. Standard fees; no 500-person cap, member discount or permanent fee exemption. Q133 pending.</v>
+        <v>Q132–133 approved: Founders tag lasts for eligible account life. Benefits conditional; eligibility/cap pending. Standard fees.</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="27.75" customHeight="1">
@@ -13899,8 +13899,8 @@
       <c r="C100" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D100" s="8" t="s">
-        <v>236</v>
+      <c r="D100" s="8" t="str">
+        <v>Q147: final settlement without automatic forfeiture. Confirm provider limits and checks before live use. PLAN §20.</v>
       </c>
     </row>
     <row r="101" spans="1:4" ht="15.75" customHeight="1">
@@ -13934,7 +13934,7 @@
         <v>21</v>
       </c>
       <c r="D103" s="11" t="str">
-        <v>Q28 approved: proportionate dispute handling; protect good-faith disputes. Review/build/tests pending. PLAN.md §20.</v>
+        <v>Q139: reverse shares; protect earned pay for platform errors. Q28 safeguards. Build/review pending. PLAN §20.</v>
       </c>
     </row>
     <row r="104" spans="1:4" ht="27.75" customHeight="1">
@@ -14088,7 +14088,7 @@
         <v>21</v>
       </c>
       <c r="D115" s="11" t="str">
-        <v>Programme direction approved Q132; eligibility, cap and duration pending Q133. No implementation yet.</v>
+        <v>Q133: lasting eligible-account tag; conditional benefits. Eligibility/cap and implementation pending.</v>
       </c>
     </row>
     <row r="116" spans="1:4" ht="15.75" customHeight="1">
@@ -24852,17 +24852,17 @@
         <v>808</v>
       </c>
       <c r="L52" s="62" t="str">
-        <v>Founder questionnaire review; commissioned draft pending</v>
+        <v>Suzanne response and commissioned drafts</v>
       </c>
       <c r="M52" s="62" t="str">
-        <v>Review Q133 Founders duration and eligibility. Q132 benefits approved; exact placements and event/prize terms pending. PLAN.md §20.</v>
+        <v>Review Suzanne response and drafts when received. Resolve flagged legal/provider points before final approval. PLAN §20.</v>
       </c>
       <c r="N52" s="63"/>
       <c r="O52" s="62" t="str">
-        <v>Q132 approved Sept 22; Q133 pending. PLAN.md §20. Suzanne Lawyer bundle, Expense Tracker row 11; commissioned terms pending.</v>
+        <v>Founder confirmed final questionnaire corrections; awaiting Suzanne Sept 23. Expense Tracker row 11 paid bundle; legal approval pending.</v>
       </c>
       <c r="P52" s="63" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="Q52" s="62" t="s">
         <v>55</v>
@@ -26740,11 +26740,11 @@
       </c>
       <c r="L87" s="62"/>
       <c r="M87" s="62" t="str">
-        <v>Define eligibility and duration after Q133. Plan Founders tag, Connect filter or Explore section, SFW Discord events and future event priority.</v>
+        <v>Finalize eligibility and enrollment cutoff/cap. Implement Q133 account-lifetime tag and conditional discovery/events; prize budgets remain separate.</v>
       </c>
       <c r="N87" s="63"/>
       <c r="O87" s="62" t="str">
-        <v>Q132 approved Sept 22. PLAN.md §20 supersedes commission-free/cost-recovery terms; Q133 pending.</v>
+        <v>Q132/Q133 approved Sept 22. PLAN.md section 20. Eligibility and event details pending.</v>
       </c>
       <c r="P87" s="63" t="n">
         <v>46287</v>
@@ -26753,7 +26753,7 @@
         <v>Founders tag; Connect filter or Explore section below top sections; SFW Discord events; future event priority. No special commission.</v>
       </c>
       <c r="R87" s="62" t="str">
-        <v>No fixed cohort, permanent ranking, member discount or Plus promise. Cash prizes optional and separately budgeted. Implementation not started.</v>
+        <v>Q133 approved: eligible account-lifetime tag; discovery/events follow terms and availability. No permanent ranking or recurring prizes. Build pending.</v>
       </c>
       <c r="S87" s="62" t="s">
         <v>1072</v>
@@ -27216,19 +27216,21 @@
       <c r="L96" s="62" t="s">
         <v>1010</v>
       </c>
-      <c r="M96" s="62" t="s">
-        <v>970</v>
+      <c r="M96" s="62" t="str">
+        <v>Design payout flow under Q134–147: eligibility, holds, fees and final settlement, including below-minimum balances. Confirm providers.</v>
       </c>
       <c r="N96" s="63"/>
-      <c r="O96" s="62"/>
-      <c r="P96" s="63">
-        <v>46250.666666666664</v>
+      <c r="O96" s="62" t="str">
+        <v>Q147 approved Sept 22, 2026. PLAN §§3.8,20; earlier payout policies retained. Provider details and implementation pending.</v>
+      </c>
+      <c r="P96" s="63" t="n">
+        <v>46287</v>
       </c>
       <c r="Q96" s="62" t="s">
         <v>235</v>
       </c>
-      <c r="R96" s="62" t="s">
-        <v>236</v>
+      <c r="R96" s="62" t="str">
+        <v>Approved policy only. Preserve payable balances after closure; final methods, fees and below-minimum resolution need legal/provider review.</v>
       </c>
       <c r="S96" s="62" t="s">
         <v>1228</v>
@@ -27325,14 +27327,14 @@
         <v>997</v>
       </c>
       <c r="M98" s="62" t="str">
-        <v>Review Q28 with counsel/processor; define trusted dispute events, then implement and test transaction access, proportionate restrictions, authorized operations and audit. PLAN.md §20.</v>
+        <v>Implement Q28/Q139 after legal/provider review: verified events, share reversals, platform-error protection, recovery, appeals and audit.</v>
       </c>
       <c r="N98" s="63"/>
       <c r="O98" s="62" t="str">
-        <v>Founder approval Sept 14, 2026; PLAN.md §20 Q28; CFPB dispute guidance and Fansly/LoyalFans policy references recorded there.</v>
+        <v>Q28 approved Sept 14; Q139 approved Sept 22, 2026. PLAN §20. Provider review and build/tests pending.</v>
       </c>
       <c r="P98" s="63" t="n">
-        <v>46279</v>
+        <v>46287</v>
       </c>
       <c r="Q98" s="62" t="s">
         <v>240</v>
@@ -27484,11 +27486,11 @@
         <v>997</v>
       </c>
       <c r="M101" s="62" t="str">
-        <v>Model actual processing, taxes, refunds, chargebacks, payout timing and operating costs against Q131. Include optional Founders event budgets.</v>
+        <v>Model Q131 and Q139–141 allocations using actual provider costs, including failed recoveries and optional Founders event budgets.</v>
       </c>
       <c r="N101" s="63"/>
       <c r="O101" s="62" t="str">
-        <v>Q131/Q132 approved. See PLAN.md section 20.</v>
+        <v>Q131/Q132/Q139–141 approved Sept 22, 2026. Actual provider fees and cost validation remain pending. PLAN §§3.8,20.</v>
       </c>
       <c r="P101" s="63" t="n">
         <v>46287</v>
@@ -28842,7 +28844,7 @@
         <v>1203</v>
       </c>
       <c r="M127" s="62" t="str">
-        <v>After Q133 terms and private-operations gates, implement Founders eligibility and badge management. No fixed cohort cap assumed.</v>
+        <v>After cohort rules and private-operations gates, implement Q133 Founders eligibility and account-lifetime tag management. No fixed cap assumed.</v>
       </c>
       <c r="N127" s="63"/>
       <c r="O127" s="62"/>
@@ -28853,7 +28855,7 @@
         <v>Manage Founders eligibility and badge assignment. Enforce a cohort limit only if approved.</v>
       </c>
       <c r="R127" s="62" t="str">
-        <v>Q132 programme direction approved; Q133 eligibility/duration pending. No member discount or separate Founders rate.</v>
+        <v>Q132–133 approved: tag lasts for eligible account life; conditional benefits. Eligibility/cap pending. No member discount or special rate.</v>
       </c>
       <c r="S127" s="62" t="s">
         <v>1260</v>

</xml_diff>